<commit_message>
Fix Japanese auxiliary verb table
</commit_message>
<xml_diff>
--- a/Studymaterials/日本語助動詞一覧.xlsx
+++ b/Studymaterials/日本語助動詞一覧.xlsx
@@ -928,7 +928,7 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>させる</t>
+          <t>しめる</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="S2" s="8" t="inlineStr">
         <is>
-          <t>たい</t>
+          <t>たがる</t>
         </is>
       </c>
       <c r="T2" s="8" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="U2" s="8" t="inlineStr">
         <is>
-          <t>ている</t>
+          <t>てある</t>
         </is>
       </c>
       <c r="V2" s="8" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>させ</t>
+          <t>しめ</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="S4" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>たがら/たがろ</t>
         </is>
       </c>
       <c r="T4" s="10" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="U4" s="10" t="inlineStr">
         <is>
-          <t>い</t>
+          <t>あら/あろ</t>
         </is>
       </c>
       <c r="V4" s="10" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>させ</t>
+          <t>しめ</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="S5" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>たがり/たがっ</t>
         </is>
       </c>
       <c r="T5" s="10" t="inlineStr">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="U5" s="10" t="inlineStr">
         <is>
-          <t>い</t>
+          <t>あり/あっ</t>
         </is>
       </c>
       <c r="V5" s="10" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>させる</t>
+          <t>しめる</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="S6" s="10" t="inlineStr">
         <is>
-          <t>たい</t>
+          <t>たがる</t>
         </is>
       </c>
       <c r="T6" s="10" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="U6" s="10" t="inlineStr">
         <is>
-          <t>いる</t>
+          <t>ある</t>
         </is>
       </c>
       <c r="V6" s="10" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>させる</t>
+          <t>しめる</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="S7" s="10" t="inlineStr">
         <is>
-          <t>たい</t>
+          <t>たがる</t>
         </is>
       </c>
       <c r="T7" s="10" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="U7" s="10" t="inlineStr">
         <is>
-          <t>いる</t>
+          <t>ある</t>
         </is>
       </c>
       <c r="V7" s="10" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>させれ</t>
+          <t>しめれ</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>たがれ</t>
         </is>
       </c>
       <c r="T8" s="10" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="U8" s="10" t="inlineStr">
         <is>
-          <t>いれ</t>
+          <t>あれ</t>
         </is>
       </c>
       <c r="V8" s="10" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>させろ</t>
+          <t>しめろ</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="S9" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>たがれ</t>
         </is>
       </c>
       <c r="T9" s="13" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="U9" s="13" t="inlineStr">
         <is>
-          <t>いろ</t>
+          <t>あれ</t>
         </is>
       </c>
       <c r="V9" s="13" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
-          <t>なら</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L12" s="21" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="K17" s="23" t="inlineStr">
         <is>
-          <t>なれ</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L17" s="23" t="inlineStr">
@@ -3212,10 +3212,10 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B1:D1"/>
-    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="E1:F1"/>
     <mergeCell ref="T1:U1"/>
     <mergeCell ref="H1:I1"/>
-    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="V1:W1"/>
     <mergeCell ref="L1:M1"/>
     <mergeCell ref="R1:S1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Polish Japanese auxiliary verb print layout
</commit_message>
<xml_diff>
--- a/Studymaterials/日本語助動詞一覧.xlsx
+++ b/Studymaterials/日本語助動詞一覧.xlsx
@@ -9,9 +9,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Sheet1'!$1:$1,'Sheet1'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1'!$A$1:$AB$17</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,14 +28,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Yu Gothic"/>
-      <charset val="128"/>
-      <family val="3"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="6.5"/>
-    </font>
-    <font>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <family val="3"/>
@@ -45,16 +38,7 @@
       <name val="Yu Gothic"/>
       <charset val="128"/>
       <family val="3"/>
-      <b val="1"/>
       <color rgb="FF000000"/>
-      <sz val="6.5"/>
-    </font>
-    <font>
-      <name val="Yu Gothic"/>
-      <charset val="128"/>
-      <family val="3"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
       <sz val="7"/>
     </font>
     <font>
@@ -63,7 +47,7 @@
       <family val="3"/>
       <b val="1"/>
       <color rgb="FF000000"/>
-      <sz val="7"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
@@ -72,23 +56,29 @@
       <color rgb="FF000000"/>
       <sz val="7"/>
     </font>
+    <font>
+      <name val="Noto Sans JP"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF404040"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -103,6 +93,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -342,76 +337,85 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -780,785 +784,792 @@
   <dimension ref="A1:AB17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13"/>
   <cols>
-    <col width="3.26953125" customWidth="1" min="1" max="1"/>
-    <col width="2" customWidth="1" min="2" max="6"/>
-    <col width="6.54296875" customWidth="1" min="7" max="8"/>
-    <col width="5.36328125" customWidth="1" min="9" max="9"/>
-    <col width="2" customWidth="1" min="10" max="13"/>
-    <col width="5.36328125" customWidth="1" min="14" max="14"/>
-    <col width="2" customWidth="1" min="15" max="16"/>
-    <col width="2.26953125" customWidth="1" min="17" max="17"/>
-    <col width="5.36328125" customWidth="1" min="18" max="19"/>
-    <col width="2.26953125" customWidth="1" min="20" max="20"/>
-    <col width="5.36328125" customWidth="1" min="21" max="21"/>
-    <col width="2" customWidth="1" min="22" max="23"/>
-    <col width="5.36328125" customWidth="1" min="24" max="24"/>
-    <col width="2" customWidth="1" min="25" max="25"/>
-    <col width="2.26953125" customWidth="1" min="26" max="26"/>
-    <col width="5.36328125" customWidth="1" min="27" max="27"/>
-    <col width="2" customWidth="1" min="28" max="28"/>
+    <col width="4.81640625" customWidth="1" min="1" max="1"/>
+    <col width="4.6328125" customWidth="1" min="2" max="6"/>
+    <col width="7.453125" customWidth="1" min="7" max="8"/>
+    <col width="5.6328125" customWidth="1" min="9" max="9"/>
+    <col width="4.6328125" customWidth="1" min="10" max="13"/>
+    <col width="5.6328125" customWidth="1" min="14" max="15"/>
+    <col width="4.6328125" customWidth="1" min="16" max="17"/>
+    <col width="5.6328125" customWidth="1" min="18" max="19"/>
+    <col width="4.6328125" customWidth="1" min="20" max="20"/>
+    <col width="5.6328125" customWidth="1" min="21" max="21"/>
+    <col width="4.6328125" customWidth="1" min="22" max="23"/>
+    <col width="5.6328125" customWidth="1" min="24" max="24"/>
+    <col width="4.6328125" customWidth="1" min="25" max="26"/>
+    <col width="5.6328125" customWidth="1" min="27" max="27"/>
+    <col width="4.6328125" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
-    <row r="1" ht="76" customHeight="1" thickBot="1">
+    <row r="1" ht="67" customHeight="1" thickBot="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>分類</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>使役</t>
         </is>
       </c>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="4" t="n"/>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>受身/尊敬/
-可能/自発</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="n"/>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="C1" s="26" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="25" t="inlineStr">
+        <is>
+          <t>受身
+尊敬
+可能
+自発</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="25" t="inlineStr">
         <is>
           <t>尊敬</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="25" t="inlineStr">
         <is>
           <t>断定</t>
         </is>
       </c>
-      <c r="I1" s="4" t="n"/>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="25" t="inlineStr">
         <is>
           <t>比況</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="K1" s="25" t="inlineStr">
         <is>
           <t>伝聞</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="L1" s="25" t="inlineStr">
         <is>
           <t>推定</t>
         </is>
       </c>
-      <c r="M1" s="4" t="n"/>
-      <c r="N1" s="5" t="inlineStr">
-        <is>
-          <t>当然/推量</t>
-        </is>
-      </c>
-      <c r="O1" s="5" t="inlineStr">
-        <is>
-          <t>意志/推量</t>
-        </is>
-      </c>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="M1" s="27" t="n"/>
+      <c r="N1" s="25" t="inlineStr">
+        <is>
+          <t>当然
+推量</t>
+        </is>
+      </c>
+      <c r="O1" s="25" t="inlineStr">
+        <is>
+          <t>意志
+推量</t>
+        </is>
+      </c>
+      <c r="P1" s="25" t="inlineStr">
         <is>
           <t>現在推量</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="Q1" s="25" t="inlineStr">
         <is>
           <t>過去推量</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="R1" s="25" t="inlineStr">
         <is>
           <t>希望</t>
         </is>
       </c>
-      <c r="S1" s="4" t="n"/>
-      <c r="T1" s="5" t="inlineStr">
+      <c r="S1" s="27" t="n"/>
+      <c r="T1" s="25" t="inlineStr">
         <is>
           <t>存続</t>
         </is>
       </c>
-      <c r="U1" s="4" t="n"/>
-      <c r="V1" s="5" t="inlineStr">
+      <c r="U1" s="27" t="n"/>
+      <c r="V1" s="25" t="inlineStr">
         <is>
           <t>完了</t>
         </is>
       </c>
-      <c r="W1" s="4" t="n"/>
-      <c r="X1" s="5" t="inlineStr">
-        <is>
-          <t>過去/詠嘆</t>
-        </is>
-      </c>
-      <c r="Y1" s="5" t="inlineStr">
+      <c r="W1" s="27" t="n"/>
+      <c r="X1" s="25" t="inlineStr">
+        <is>
+          <t>過去
+詠嘆</t>
+        </is>
+      </c>
+      <c r="Y1" s="25" t="inlineStr">
         <is>
           <t>過去</t>
         </is>
       </c>
-      <c r="Z1" s="5" t="inlineStr">
+      <c r="Z1" s="25" t="inlineStr">
         <is>
           <t>打消推量</t>
         </is>
       </c>
-      <c r="AA1" s="5" t="inlineStr">
+      <c r="AA1" s="25" t="inlineStr">
         <is>
           <t>打消</t>
         </is>
       </c>
-      <c r="AB1" s="6" t="inlineStr">
+      <c r="AB1" s="3" t="inlineStr">
         <is>
           <t>禁止</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="51" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
+    <row r="2" ht="76" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>現代口語</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>せる</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>させる</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>しめる</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>れる</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>られる</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>なさる</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>だ</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>である</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>ようだ</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>そうだ</t>
         </is>
       </c>
-      <c r="L2" s="8" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>ようだ</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>らしい</t>
         </is>
       </c>
-      <c r="N2" s="8" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>だろう
 はずだ</t>
         </is>
       </c>
-      <c r="O2" s="8" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>だろう</t>
         </is>
       </c>
-      <c r="P2" s="8" t="inlineStr">
+      <c r="P2" s="6" t="inlineStr">
         <is>
           <t>︴だろう</t>
         </is>
       </c>
-      <c r="Q2" s="8" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
         <is>
           <t>︴ただろう</t>
         </is>
       </c>
-      <c r="R2" s="8" t="inlineStr">
+      <c r="R2" s="5" t="inlineStr">
         <is>
           <t>たい</t>
         </is>
       </c>
-      <c r="S2" s="8" t="inlineStr">
+      <c r="S2" s="5" t="inlineStr">
         <is>
           <t>たがる</t>
         </is>
       </c>
-      <c r="T2" s="8" t="inlineStr">
+      <c r="T2" s="5" t="inlineStr">
         <is>
           <t>ている</t>
         </is>
       </c>
-      <c r="U2" s="8" t="inlineStr">
+      <c r="U2" s="5" t="inlineStr">
         <is>
           <t>てある</t>
         </is>
       </c>
-      <c r="V2" s="8" t="inlineStr">
+      <c r="V2" s="5" t="inlineStr">
         <is>
           <t>た</t>
         </is>
       </c>
-      <c r="W2" s="8" t="inlineStr">
+      <c r="W2" s="5" t="inlineStr">
         <is>
           <t>た</t>
         </is>
       </c>
-      <c r="X2" s="8" t="inlineStr">
+      <c r="X2" s="5" t="inlineStr">
         <is>
           <t>た
 だ</t>
         </is>
       </c>
-      <c r="Y2" s="8" t="inlineStr">
+      <c r="Y2" s="5" t="inlineStr">
         <is>
           <t>た</t>
         </is>
       </c>
-      <c r="Z2" s="8" t="inlineStr">
+      <c r="Z2" s="6" t="inlineStr">
         <is>
           <t>︴ないだろう</t>
         </is>
       </c>
-      <c r="AA2" s="8" t="inlineStr">
+      <c r="AA2" s="5" t="inlineStr">
         <is>
           <t>ない</t>
         </is>
       </c>
-      <c r="AB2" s="9" t="inlineStr">
+      <c r="AB2" s="7" t="inlineStr">
         <is>
           <t>︴するな</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="41" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+    <row r="3" ht="51" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>接続</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>体言
 連体形</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>体言
 連体形</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>連体形</t>
         </is>
       </c>
-      <c r="K3" s="10" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>連体形</t>
         </is>
       </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="N3" s="10" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="O3" s="10" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="P3" s="10" t="inlineStr">
+      <c r="P3" s="8" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="Q3" s="10" t="inlineStr">
+      <c r="Q3" s="8" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="R3" s="10" t="inlineStr">
+      <c r="R3" s="8" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="S3" s="10" t="inlineStr">
+      <c r="S3" s="8" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="T3" s="10" t="inlineStr">
+      <c r="T3" s="8" t="inlineStr">
         <is>
           <t>連用形＋て</t>
         </is>
       </c>
-      <c r="U3" s="10" t="inlineStr">
+      <c r="U3" s="8" t="inlineStr">
         <is>
           <t>連用形＋て</t>
         </is>
       </c>
-      <c r="V3" s="10" t="inlineStr">
+      <c r="V3" s="8" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="W3" s="10" t="inlineStr">
+      <c r="W3" s="8" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="X3" s="10" t="inlineStr">
+      <c r="X3" s="8" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="Y3" s="10" t="inlineStr">
+      <c r="Y3" s="8" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="Z3" s="10" t="inlineStr">
+      <c r="Z3" s="8" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="AA3" s="10" t="inlineStr">
+      <c r="AA3" s="8" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="AB3" s="11" t="inlineStr">
+      <c r="AB3" s="9" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="55" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+    <row r="4" ht="61" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>せ</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>させ</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>しめ</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>れ</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>られ</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>なさら
 なさろ</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>だろ</t>
         </is>
       </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J4" s="10" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>ようだろ</t>
         </is>
       </c>
-      <c r="K4" s="10" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>そうだろ</t>
         </is>
       </c>
-      <c r="L4" s="10" t="inlineStr">
+      <c r="L4" s="8" t="inlineStr">
         <is>
           <t>ようだろ</t>
         </is>
       </c>
-      <c r="M4" s="10" t="inlineStr">
+      <c r="M4" s="8" t="inlineStr">
         <is>
           <t>らしかろ</t>
         </is>
       </c>
-      <c r="N4" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O4" s="10" t="inlineStr">
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
         <is>
           <t>だろ</t>
         </is>
       </c>
-      <c r="P4" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q4" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" s="10" t="inlineStr">
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
         <is>
           <t>たかろ</t>
         </is>
       </c>
-      <c r="S4" s="10" t="inlineStr">
-        <is>
-          <t>たがら/たがろ</t>
-        </is>
-      </c>
-      <c r="T4" s="10" t="inlineStr">
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>たがら
+たがろ</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="inlineStr">
         <is>
           <t>い</t>
         </is>
       </c>
-      <c r="U4" s="10" t="inlineStr">
-        <is>
-          <t>あら/あろ</t>
-        </is>
-      </c>
-      <c r="V4" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W4" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X4" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y4" s="10" t="inlineStr">
+      <c r="U4" s="8" t="inlineStr">
+        <is>
+          <t>あら
+あろ</t>
+        </is>
+      </c>
+      <c r="V4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y4" s="8" t="inlineStr">
         <is>
           <t>たろ</t>
         </is>
       </c>
-      <c r="Z4" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA4" s="10" t="inlineStr">
+      <c r="Z4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA4" s="8" t="inlineStr">
         <is>
           <t>なかろ</t>
         </is>
       </c>
-      <c r="AB4" s="11" t="inlineStr">
+      <c r="AB4" s="9" t="inlineStr">
         <is>
           <t>な</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="55" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="5" ht="81" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>せ</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>させ</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>しめ</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>れ</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>られ</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>なさり
 なさっ
 なさい</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>だっ
 で
 に</t>
         </is>
       </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>ようで</t>
         </is>
       </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>そうで</t>
         </is>
       </c>
-      <c r="L5" s="10" t="inlineStr">
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>ようで</t>
         </is>
       </c>
-      <c r="M5" s="10" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>らしく</t>
         </is>
       </c>
-      <c r="N5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" s="10" t="inlineStr">
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
         <is>
           <t>たく</t>
         </is>
       </c>
-      <c r="S5" s="10" t="inlineStr">
-        <is>
-          <t>たがり/たがっ</t>
-        </is>
-      </c>
-      <c r="T5" s="10" t="inlineStr">
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>たがり
+たがっ</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
         <is>
           <t>い</t>
         </is>
       </c>
-      <c r="U5" s="10" t="inlineStr">
-        <is>
-          <t>あり/あっ</t>
-        </is>
-      </c>
-      <c r="V5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y5" s="10" t="inlineStr">
+      <c r="U5" s="8" t="inlineStr">
+        <is>
+          <t>あり
+あっ</t>
+        </is>
+      </c>
+      <c r="V5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y5" s="8" t="inlineStr">
         <is>
           <t>た</t>
         </is>
       </c>
-      <c r="Z5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA5" s="10" t="inlineStr">
+      <c r="Z5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA5" s="8" t="inlineStr">
         <is>
           <t>なく</t>
         </is>
       </c>
-      <c r="AB5" s="11" t="inlineStr">
+      <c r="AB5" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="55" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+    <row r="6" ht="83" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>せる</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>させる</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>しめる</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>れる</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>られる</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>なさる</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>だ</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>である</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>ようだ</t>
         </is>
       </c>
-      <c r="K6" s="10" t="inlineStr">
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>そうだ</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="L6" s="8" t="inlineStr">
         <is>
           <t>ようだ</t>
         </is>
       </c>
-      <c r="M6" s="10" t="inlineStr">
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>らしい</t>
         </is>
       </c>
-      <c r="N6" s="10" t="inlineStr">
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>だろう</t>
         </is>
       </c>
-      <c r="O6" s="10" t="inlineStr">
+      <c r="O6" s="8" t="inlineStr">
         <is>
           <t>だろう</t>
         </is>
@@ -1573,43 +1584,43 @@
           <t>︴ただろう</t>
         </is>
       </c>
-      <c r="R6" s="10" t="inlineStr">
+      <c r="R6" s="8" t="inlineStr">
         <is>
           <t>たい</t>
         </is>
       </c>
-      <c r="S6" s="10" t="inlineStr">
+      <c r="S6" s="8" t="inlineStr">
         <is>
           <t>たがる</t>
         </is>
       </c>
-      <c r="T6" s="10" t="inlineStr">
+      <c r="T6" s="8" t="inlineStr">
         <is>
           <t>いる</t>
         </is>
       </c>
-      <c r="U6" s="10" t="inlineStr">
+      <c r="U6" s="8" t="inlineStr">
         <is>
           <t>ある</t>
         </is>
       </c>
-      <c r="V6" s="10" t="inlineStr">
+      <c r="V6" s="8" t="inlineStr">
         <is>
           <t>た</t>
         </is>
       </c>
-      <c r="W6" s="10" t="inlineStr">
+      <c r="W6" s="8" t="inlineStr">
         <is>
           <t>た</t>
         </is>
       </c>
-      <c r="X6" s="10" t="inlineStr">
+      <c r="X6" s="8" t="inlineStr">
         <is>
           <t>た
 だ</t>
         </is>
       </c>
-      <c r="Y6" s="10" t="inlineStr">
+      <c r="Y6" s="8" t="inlineStr">
         <is>
           <t>た</t>
         </is>
@@ -1619,89 +1630,89 @@
           <t>︴ないだろう</t>
         </is>
       </c>
-      <c r="AA6" s="10" t="inlineStr">
+      <c r="AA6" s="8" t="inlineStr">
         <is>
           <t>ない</t>
         </is>
       </c>
-      <c r="AB6" s="11" t="inlineStr">
+      <c r="AB6" s="9" t="inlineStr">
         <is>
           <t>な</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="55" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="7" ht="83" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>連体形</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>せる</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>させる</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>しめる</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>れる</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>られる</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>なさる</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>な</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>である</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>ような</t>
         </is>
       </c>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>そうな</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="L7" s="8" t="inlineStr">
         <is>
           <t>ような</t>
         </is>
       </c>
-      <c r="M7" s="10" t="inlineStr">
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t>らしい</t>
         </is>
       </c>
-      <c r="N7" s="10" t="inlineStr">
+      <c r="N7" s="8" t="inlineStr">
         <is>
           <t>だろう</t>
         </is>
       </c>
-      <c r="O7" s="10" t="inlineStr">
+      <c r="O7" s="8" t="inlineStr">
         <is>
           <t>だろう</t>
         </is>
@@ -1716,43 +1727,43 @@
           <t>︴ただろう</t>
         </is>
       </c>
-      <c r="R7" s="10" t="inlineStr">
+      <c r="R7" s="8" t="inlineStr">
         <is>
           <t>たい</t>
         </is>
       </c>
-      <c r="S7" s="10" t="inlineStr">
+      <c r="S7" s="8" t="inlineStr">
         <is>
           <t>たがる</t>
         </is>
       </c>
-      <c r="T7" s="10" t="inlineStr">
+      <c r="T7" s="8" t="inlineStr">
         <is>
           <t>いる</t>
         </is>
       </c>
-      <c r="U7" s="10" t="inlineStr">
+      <c r="U7" s="8" t="inlineStr">
         <is>
           <t>ある</t>
         </is>
       </c>
-      <c r="V7" s="10" t="inlineStr">
+      <c r="V7" s="8" t="inlineStr">
         <is>
           <t>た</t>
         </is>
       </c>
-      <c r="W7" s="10" t="inlineStr">
+      <c r="W7" s="8" t="inlineStr">
         <is>
           <t>た</t>
         </is>
       </c>
-      <c r="X7" s="10" t="inlineStr">
+      <c r="X7" s="8" t="inlineStr">
         <is>
           <t>た
 だ</t>
         </is>
       </c>
-      <c r="Y7" s="10" t="inlineStr">
+      <c r="Y7" s="8" t="inlineStr">
         <is>
           <t>た</t>
         </is>
@@ -1762,59 +1773,59 @@
           <t>︴ないだろう</t>
         </is>
       </c>
-      <c r="AA7" s="10" t="inlineStr">
+      <c r="AA7" s="8" t="inlineStr">
         <is>
           <t>ない</t>
         </is>
       </c>
-      <c r="AB7" s="11" t="inlineStr">
+      <c r="AB7" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="55" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+    <row r="8" ht="65" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>仮定形</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>せれ</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>させれ</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>しめれ</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>れれ</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>られれ</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>なされ</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>なら</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>であれ</t>
         </is>
@@ -1839,1371 +1850,1371 @@
           <t>らしけれ</t>
         </is>
       </c>
-      <c r="N8" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O8" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P8" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q8" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R8" s="10" t="inlineStr">
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
         <is>
           <t>たけれ</t>
         </is>
       </c>
-      <c r="S8" s="10" t="inlineStr">
+      <c r="S8" s="8" t="inlineStr">
         <is>
           <t>たがれ</t>
         </is>
       </c>
-      <c r="T8" s="10" t="inlineStr">
+      <c r="T8" s="8" t="inlineStr">
         <is>
           <t>いれ</t>
         </is>
       </c>
-      <c r="U8" s="10" t="inlineStr">
+      <c r="U8" s="8" t="inlineStr">
         <is>
           <t>あれ</t>
         </is>
       </c>
-      <c r="V8" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W8" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X8" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y8" s="10" t="inlineStr">
+      <c r="V8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y8" s="8" t="inlineStr">
         <is>
           <t>たら</t>
         </is>
       </c>
-      <c r="Z8" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA8" s="10" t="inlineStr">
+      <c r="Z8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA8" s="8" t="inlineStr">
         <is>
           <t>なけれ</t>
         </is>
       </c>
-      <c r="AB8" s="11" t="inlineStr">
+      <c r="AB8" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1" thickBot="1">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="59" customHeight="1" thickBot="1">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>命令形</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>せろ</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>させろ</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>しめろ</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>れろ</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>られろ</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>なさい
 なされ</t>
         </is>
       </c>
-      <c r="H9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S9" s="13" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" s="12" t="inlineStr">
         <is>
           <t>たがれ</t>
         </is>
       </c>
-      <c r="T9" s="13" t="inlineStr">
+      <c r="T9" s="12" t="inlineStr">
         <is>
           <t>いろ</t>
         </is>
       </c>
-      <c r="U9" s="13" t="inlineStr">
+      <c r="U9" s="12" t="inlineStr">
         <is>
           <t>あれ</t>
         </is>
       </c>
-      <c r="V9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB9" s="14" t="inlineStr">
+      <c r="V9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB9" s="13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1" thickBot="1">
-      <c r="A10" s="15" t="inlineStr">
+    <row r="10" ht="55" customHeight="1" thickBot="1">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>文語</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>す</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>さす</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>しむ</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>る</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>らる</t>
         </is>
       </c>
-      <c r="G10" s="16" t="inlineStr">
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>給ふ</t>
         </is>
       </c>
-      <c r="H10" s="16" t="inlineStr">
+      <c r="H10" s="14" t="inlineStr">
         <is>
           <t>なり</t>
         </is>
       </c>
-      <c r="I10" s="16" t="inlineStr">
+      <c r="I10" s="14" t="inlineStr">
         <is>
           <t>たり</t>
         </is>
       </c>
-      <c r="J10" s="16" t="inlineStr">
+      <c r="J10" s="14" t="inlineStr">
         <is>
           <t>ごとし</t>
         </is>
       </c>
-      <c r="K10" s="16" t="inlineStr">
+      <c r="K10" s="14" t="inlineStr">
         <is>
           <t>なり</t>
         </is>
       </c>
-      <c r="L10" s="16" t="inlineStr">
+      <c r="L10" s="14" t="inlineStr">
         <is>
           <t>めり</t>
         </is>
       </c>
-      <c r="M10" s="16" t="inlineStr">
+      <c r="M10" s="14" t="inlineStr">
         <is>
           <t>らし</t>
         </is>
       </c>
-      <c r="N10" s="16" t="inlineStr">
+      <c r="N10" s="14" t="inlineStr">
         <is>
           <t>べし</t>
         </is>
       </c>
-      <c r="O10" s="16" t="inlineStr">
+      <c r="O10" s="14" t="inlineStr">
         <is>
           <t>む</t>
         </is>
       </c>
-      <c r="P10" s="16" t="inlineStr">
+      <c r="P10" s="14" t="inlineStr">
         <is>
           <t>らむ</t>
         </is>
       </c>
-      <c r="Q10" s="16" t="inlineStr">
+      <c r="Q10" s="14" t="inlineStr">
         <is>
           <t>けむ</t>
         </is>
       </c>
-      <c r="R10" s="16" t="inlineStr">
+      <c r="R10" s="14" t="inlineStr">
         <is>
           <t>たし</t>
         </is>
       </c>
-      <c r="S10" s="16" t="inlineStr">
+      <c r="S10" s="14" t="inlineStr">
         <is>
           <t>まほし</t>
         </is>
       </c>
-      <c r="T10" s="16" t="inlineStr">
+      <c r="T10" s="14" t="inlineStr">
         <is>
           <t>たり</t>
         </is>
       </c>
-      <c r="U10" s="16" t="inlineStr">
+      <c r="U10" s="14" t="inlineStr">
         <is>
           <t>り</t>
         </is>
       </c>
-      <c r="V10" s="16" t="inlineStr">
+      <c r="V10" s="14" t="inlineStr">
         <is>
           <t>つ</t>
         </is>
       </c>
-      <c r="W10" s="16" t="inlineStr">
+      <c r="W10" s="14" t="inlineStr">
         <is>
           <t>ぬ</t>
         </is>
       </c>
-      <c r="X10" s="16" t="inlineStr">
+      <c r="X10" s="14" t="inlineStr">
         <is>
           <t>けり</t>
         </is>
       </c>
-      <c r="Y10" s="16" t="inlineStr">
+      <c r="Y10" s="14" t="inlineStr">
         <is>
           <t>き</t>
         </is>
       </c>
-      <c r="Z10" s="16" t="inlineStr">
+      <c r="Z10" s="14" t="inlineStr">
         <is>
           <t>じ</t>
         </is>
       </c>
-      <c r="AA10" s="16" t="inlineStr">
+      <c r="AA10" s="14" t="inlineStr">
         <is>
           <t>ず</t>
         </is>
       </c>
-      <c r="AB10" s="17" t="inlineStr">
+      <c r="AB10" s="15" t="inlineStr">
         <is>
           <t>な</t>
         </is>
       </c>
     </row>
     <row r="11" ht="53" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>接続</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="F11" s="19" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="G11" s="19" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="H11" s="19" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>体言
 連体形</t>
         </is>
       </c>
-      <c r="I11" s="19" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>体言
 連体形</t>
         </is>
       </c>
-      <c r="J11" s="19" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>連体形</t>
         </is>
       </c>
-      <c r="K11" s="19" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="L11" s="19" t="inlineStr">
+      <c r="L11" s="17" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="M11" s="19" t="inlineStr">
+      <c r="M11" s="17" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="N11" s="19" t="inlineStr">
+      <c r="N11" s="17" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="O11" s="19" t="inlineStr">
+      <c r="O11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="P11" s="19" t="inlineStr">
+      <c r="P11" s="17" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="Q11" s="19" t="inlineStr">
+      <c r="Q11" s="17" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="R11" s="19" t="inlineStr">
+      <c r="R11" s="17" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="S11" s="19" t="inlineStr">
+      <c r="S11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="T11" s="19" t="inlineStr">
+      <c r="T11" s="17" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="U11" s="19" t="inlineStr">
+      <c r="U11" s="17" t="inlineStr">
         <is>
           <t>サ未然
 四已然</t>
         </is>
       </c>
-      <c r="V11" s="19" t="inlineStr">
+      <c r="V11" s="17" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="W11" s="19" t="inlineStr">
+      <c r="W11" s="17" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="X11" s="19" t="inlineStr">
+      <c r="X11" s="17" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="Y11" s="19" t="inlineStr">
+      <c r="Y11" s="17" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="Z11" s="19" t="inlineStr">
+      <c r="Z11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="AA11" s="19" t="inlineStr">
+      <c r="AA11" s="17" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="AB11" s="20" t="inlineStr">
+      <c r="AB11" s="18" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="65" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="12" ht="71" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>未然形</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>せ</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>させ</t>
         </is>
       </c>
-      <c r="D12" s="21" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>しめ</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>れ</t>
         </is>
       </c>
-      <c r="F12" s="21" t="inlineStr">
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>られ</t>
         </is>
       </c>
-      <c r="G12" s="21" t="inlineStr">
+      <c r="G12" s="19" t="inlineStr">
         <is>
           <t>たまは</t>
         </is>
       </c>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="H12" s="19" t="inlineStr">
         <is>
           <t>なら</t>
         </is>
       </c>
-      <c r="I12" s="21" t="inlineStr">
+      <c r="I12" s="19" t="inlineStr">
         <is>
           <t>たら</t>
         </is>
       </c>
-      <c r="J12" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K12" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L12" s="21" t="inlineStr">
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="19" t="inlineStr">
         <is>
           <t>めら</t>
         </is>
       </c>
-      <c r="M12" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N12" s="21" t="inlineStr">
+      <c r="M12" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N12" s="19" t="inlineStr">
         <is>
           <t>べく
 べから</t>
         </is>
       </c>
-      <c r="O12" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P12" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q12" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R12" s="21" t="inlineStr">
+      <c r="O12" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P12" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q12" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" s="19" t="inlineStr">
         <is>
           <t>たく
 たから</t>
         </is>
       </c>
-      <c r="S12" s="21" t="inlineStr">
+      <c r="S12" s="20" t="inlineStr">
         <is>
           <t>まほしから</t>
         </is>
       </c>
-      <c r="T12" s="21" t="inlineStr">
+      <c r="T12" s="19" t="inlineStr">
         <is>
           <t>たら</t>
         </is>
       </c>
-      <c r="U12" s="21" t="inlineStr">
+      <c r="U12" s="19" t="inlineStr">
         <is>
           <t>ら</t>
         </is>
       </c>
-      <c r="V12" s="21" t="inlineStr">
+      <c r="V12" s="19" t="inlineStr">
         <is>
           <t>て</t>
         </is>
       </c>
-      <c r="W12" s="21" t="inlineStr">
+      <c r="W12" s="19" t="inlineStr">
         <is>
           <t>な</t>
         </is>
       </c>
-      <c r="X12" s="21" t="inlineStr">
+      <c r="X12" s="19" t="inlineStr">
         <is>
           <t>けら</t>
         </is>
       </c>
-      <c r="Y12" s="21" t="inlineStr">
+      <c r="Y12" s="19" t="inlineStr">
         <is>
           <t>せ</t>
         </is>
       </c>
-      <c r="Z12" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA12" s="21" t="inlineStr">
+      <c r="Z12" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA12" s="19" t="inlineStr">
         <is>
           <t>ず
 ざら</t>
         </is>
       </c>
-      <c r="AB12" s="22" t="inlineStr">
+      <c r="AB12" s="21" t="inlineStr">
         <is>
           <t>な</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="65" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+    <row r="13" ht="81" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>連用形</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>せ</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>させ</t>
         </is>
       </c>
-      <c r="D13" s="21" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>しめ</t>
         </is>
       </c>
-      <c r="E13" s="21" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
         <is>
           <t>れ</t>
         </is>
       </c>
-      <c r="F13" s="21" t="inlineStr">
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>られ</t>
         </is>
       </c>
-      <c r="G13" s="21" t="inlineStr">
+      <c r="G13" s="19" t="inlineStr">
         <is>
           <t>たまひ</t>
         </is>
       </c>
-      <c r="H13" s="21" t="inlineStr">
+      <c r="H13" s="19" t="inlineStr">
         <is>
           <t>なり</t>
         </is>
       </c>
-      <c r="I13" s="21" t="inlineStr">
+      <c r="I13" s="19" t="inlineStr">
         <is>
           <t>たり</t>
         </is>
       </c>
-      <c r="J13" s="21" t="inlineStr">
+      <c r="J13" s="19" t="inlineStr">
         <is>
           <t>ごとく</t>
         </is>
       </c>
-      <c r="K13" s="21" t="inlineStr">
+      <c r="K13" s="19" t="inlineStr">
         <is>
           <t>なり</t>
         </is>
       </c>
-      <c r="L13" s="21" t="inlineStr">
+      <c r="L13" s="19" t="inlineStr">
         <is>
           <t>めり</t>
         </is>
       </c>
-      <c r="M13" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N13" s="21" t="inlineStr">
+      <c r="M13" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N13" s="19" t="inlineStr">
         <is>
           <t>べく
 べかり</t>
         </is>
       </c>
-      <c r="O13" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P13" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q13" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R13" s="21" t="inlineStr">
+      <c r="O13" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P13" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R13" s="19" t="inlineStr">
         <is>
           <t>たく
 たかり</t>
         </is>
       </c>
-      <c r="S13" s="21" t="inlineStr">
+      <c r="S13" s="24" t="inlineStr">
         <is>
           <t>まほしく
 まほしかり</t>
         </is>
       </c>
-      <c r="T13" s="21" t="inlineStr">
+      <c r="T13" s="19" t="inlineStr">
         <is>
           <t>たり</t>
         </is>
       </c>
-      <c r="U13" s="21" t="inlineStr">
+      <c r="U13" s="19" t="inlineStr">
         <is>
           <t>り</t>
         </is>
       </c>
-      <c r="V13" s="21" t="inlineStr">
+      <c r="V13" s="19" t="inlineStr">
         <is>
           <t>て</t>
         </is>
       </c>
-      <c r="W13" s="21" t="inlineStr">
+      <c r="W13" s="19" t="inlineStr">
         <is>
           <t>に</t>
         </is>
       </c>
-      <c r="X13" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y13" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z13" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA13" s="21" t="inlineStr">
+      <c r="X13" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y13" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z13" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA13" s="19" t="inlineStr">
         <is>
           <t>ず
 ざり</t>
         </is>
       </c>
-      <c r="AB13" s="22" t="inlineStr">
+      <c r="AB13" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="49" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="14" ht="53" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>終止形</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>す</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>さす</t>
         </is>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>しむ</t>
         </is>
       </c>
-      <c r="E14" s="21" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>る</t>
         </is>
       </c>
-      <c r="F14" s="21" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>らる</t>
         </is>
       </c>
-      <c r="G14" s="21" t="inlineStr">
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>たまふ</t>
         </is>
       </c>
-      <c r="H14" s="21" t="inlineStr">
+      <c r="H14" s="19" t="inlineStr">
         <is>
           <t>なり</t>
         </is>
       </c>
-      <c r="I14" s="21" t="inlineStr">
+      <c r="I14" s="19" t="inlineStr">
         <is>
           <t>たり</t>
         </is>
       </c>
-      <c r="J14" s="21" t="inlineStr">
+      <c r="J14" s="19" t="inlineStr">
         <is>
           <t>ごとし</t>
         </is>
       </c>
-      <c r="K14" s="21" t="inlineStr">
+      <c r="K14" s="19" t="inlineStr">
         <is>
           <t>なり</t>
         </is>
       </c>
-      <c r="L14" s="21" t="inlineStr">
+      <c r="L14" s="19" t="inlineStr">
         <is>
           <t>めり</t>
         </is>
       </c>
-      <c r="M14" s="21" t="inlineStr">
+      <c r="M14" s="19" t="inlineStr">
         <is>
           <t>らし</t>
         </is>
       </c>
-      <c r="N14" s="21" t="inlineStr">
+      <c r="N14" s="19" t="inlineStr">
         <is>
           <t>べし</t>
         </is>
       </c>
-      <c r="O14" s="21" t="inlineStr">
+      <c r="O14" s="19" t="inlineStr">
         <is>
           <t>む</t>
         </is>
       </c>
-      <c r="P14" s="21" t="inlineStr">
+      <c r="P14" s="19" t="inlineStr">
         <is>
           <t>らむ</t>
         </is>
       </c>
-      <c r="Q14" s="21" t="inlineStr">
+      <c r="Q14" s="19" t="inlineStr">
         <is>
           <t>けむ</t>
         </is>
       </c>
-      <c r="R14" s="21" t="inlineStr">
+      <c r="R14" s="19" t="inlineStr">
         <is>
           <t>たし</t>
         </is>
       </c>
-      <c r="S14" s="21" t="inlineStr">
+      <c r="S14" s="19" t="inlineStr">
         <is>
           <t>まほし</t>
         </is>
       </c>
-      <c r="T14" s="21" t="inlineStr">
+      <c r="T14" s="19" t="inlineStr">
         <is>
           <t>たり</t>
         </is>
       </c>
-      <c r="U14" s="21" t="inlineStr">
+      <c r="U14" s="19" t="inlineStr">
         <is>
           <t>り</t>
         </is>
       </c>
-      <c r="V14" s="21" t="inlineStr">
+      <c r="V14" s="19" t="inlineStr">
         <is>
           <t>つ</t>
         </is>
       </c>
-      <c r="W14" s="21" t="inlineStr">
+      <c r="W14" s="19" t="inlineStr">
         <is>
           <t>ぬ</t>
         </is>
       </c>
-      <c r="X14" s="21" t="inlineStr">
+      <c r="X14" s="19" t="inlineStr">
         <is>
           <t>けり</t>
         </is>
       </c>
-      <c r="Y14" s="21" t="inlineStr">
+      <c r="Y14" s="19" t="inlineStr">
         <is>
           <t>き</t>
         </is>
       </c>
-      <c r="Z14" s="21" t="inlineStr">
+      <c r="Z14" s="19" t="inlineStr">
         <is>
           <t>じ</t>
         </is>
       </c>
-      <c r="AA14" s="21" t="inlineStr">
+      <c r="AA14" s="19" t="inlineStr">
         <is>
           <t>ず</t>
         </is>
       </c>
-      <c r="AB14" s="22" t="inlineStr">
+      <c r="AB14" s="21" t="inlineStr">
         <is>
           <t>な</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="69" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="15" ht="81" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>連体形</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>する</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="C15" s="19" t="inlineStr">
         <is>
           <t>さする</t>
         </is>
       </c>
-      <c r="D15" s="21" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>しむる</t>
         </is>
       </c>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>るる</t>
         </is>
       </c>
-      <c r="F15" s="21" t="inlineStr">
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>らるる</t>
         </is>
       </c>
-      <c r="G15" s="21" t="inlineStr">
+      <c r="G15" s="19" t="inlineStr">
         <is>
           <t>たまふ</t>
         </is>
       </c>
-      <c r="H15" s="21" t="inlineStr">
+      <c r="H15" s="19" t="inlineStr">
         <is>
           <t>なる</t>
         </is>
       </c>
-      <c r="I15" s="21" t="inlineStr">
+      <c r="I15" s="19" t="inlineStr">
         <is>
           <t>たる</t>
         </is>
       </c>
-      <c r="J15" s="21" t="inlineStr">
+      <c r="J15" s="19" t="inlineStr">
         <is>
           <t>ごとき</t>
         </is>
       </c>
-      <c r="K15" s="21" t="inlineStr">
+      <c r="K15" s="19" t="inlineStr">
         <is>
           <t>なる</t>
         </is>
       </c>
-      <c r="L15" s="21" t="inlineStr">
+      <c r="L15" s="19" t="inlineStr">
         <is>
           <t>める</t>
         </is>
       </c>
-      <c r="M15" s="21" t="inlineStr">
+      <c r="M15" s="19" t="inlineStr">
         <is>
           <t>らし</t>
         </is>
       </c>
-      <c r="N15" s="21" t="inlineStr">
+      <c r="N15" s="19" t="inlineStr">
         <is>
           <t>べき
 べかる</t>
         </is>
       </c>
-      <c r="O15" s="21" t="inlineStr">
+      <c r="O15" s="19" t="inlineStr">
         <is>
           <t>む</t>
         </is>
       </c>
-      <c r="P15" s="21" t="inlineStr">
+      <c r="P15" s="19" t="inlineStr">
         <is>
           <t>らむ</t>
         </is>
       </c>
-      <c r="Q15" s="21" t="inlineStr">
+      <c r="Q15" s="19" t="inlineStr">
         <is>
           <t>けむ</t>
         </is>
       </c>
-      <c r="R15" s="21" t="inlineStr">
+      <c r="R15" s="19" t="inlineStr">
         <is>
           <t>たき
 たかる</t>
         </is>
       </c>
-      <c r="S15" s="21" t="inlineStr">
+      <c r="S15" s="24" t="inlineStr">
         <is>
           <t>まほしき
 まほしかる</t>
         </is>
       </c>
-      <c r="T15" s="21" t="inlineStr">
+      <c r="T15" s="19" t="inlineStr">
         <is>
           <t>たる</t>
         </is>
       </c>
-      <c r="U15" s="21" t="inlineStr">
+      <c r="U15" s="19" t="inlineStr">
         <is>
           <t>る</t>
         </is>
       </c>
-      <c r="V15" s="21" t="inlineStr">
+      <c r="V15" s="19" t="inlineStr">
         <is>
           <t>つる</t>
         </is>
       </c>
-      <c r="W15" s="21" t="inlineStr">
+      <c r="W15" s="19" t="inlineStr">
         <is>
           <t>ぬる</t>
         </is>
       </c>
-      <c r="X15" s="21" t="inlineStr">
+      <c r="X15" s="19" t="inlineStr">
         <is>
           <t>ける</t>
         </is>
       </c>
-      <c r="Y15" s="21" t="inlineStr">
+      <c r="Y15" s="19" t="inlineStr">
         <is>
           <t>し</t>
         </is>
       </c>
-      <c r="Z15" s="21" t="inlineStr">
+      <c r="Z15" s="19" t="inlineStr">
         <is>
           <t>じ</t>
         </is>
       </c>
-      <c r="AA15" s="21" t="inlineStr">
+      <c r="AA15" s="19" t="inlineStr">
         <is>
           <t>ぬ
 ざる</t>
         </is>
       </c>
-      <c r="AB15" s="22" t="inlineStr">
+      <c r="AB15" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="55" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="16" ht="71" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>已然形</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>すれ</t>
         </is>
       </c>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="C16" s="19" t="inlineStr">
         <is>
           <t>さすれ</t>
         </is>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>しむれ</t>
         </is>
       </c>
-      <c r="E16" s="21" t="inlineStr">
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>るれ</t>
         </is>
       </c>
-      <c r="F16" s="21" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>らるれ</t>
         </is>
       </c>
-      <c r="G16" s="21" t="inlineStr">
+      <c r="G16" s="19" t="inlineStr">
         <is>
           <t>たまへ</t>
         </is>
       </c>
-      <c r="H16" s="21" t="inlineStr">
+      <c r="H16" s="19" t="inlineStr">
         <is>
           <t>なれ</t>
         </is>
       </c>
-      <c r="I16" s="21" t="inlineStr">
+      <c r="I16" s="19" t="inlineStr">
         <is>
           <t>たれ</t>
         </is>
       </c>
-      <c r="J16" s="21" t="inlineStr">
+      <c r="J16" s="19" t="inlineStr">
         <is>
           <t>ごとけれ</t>
         </is>
       </c>
-      <c r="K16" s="21" t="inlineStr">
+      <c r="K16" s="19" t="inlineStr">
         <is>
           <t>なれ</t>
         </is>
       </c>
-      <c r="L16" s="21" t="inlineStr">
+      <c r="L16" s="19" t="inlineStr">
         <is>
           <t>めれ</t>
         </is>
       </c>
-      <c r="M16" s="21" t="inlineStr">
+      <c r="M16" s="19" t="inlineStr">
         <is>
           <t>らし</t>
         </is>
       </c>
-      <c r="N16" s="21" t="inlineStr">
+      <c r="N16" s="19" t="inlineStr">
         <is>
           <t>べけれ</t>
         </is>
       </c>
-      <c r="O16" s="21" t="inlineStr">
+      <c r="O16" s="19" t="inlineStr">
         <is>
           <t>め</t>
         </is>
       </c>
-      <c r="P16" s="21" t="inlineStr">
+      <c r="P16" s="19" t="inlineStr">
         <is>
           <t>らめ</t>
         </is>
       </c>
-      <c r="Q16" s="21" t="inlineStr">
+      <c r="Q16" s="19" t="inlineStr">
         <is>
           <t>けめ</t>
         </is>
       </c>
-      <c r="R16" s="21" t="inlineStr">
+      <c r="R16" s="19" t="inlineStr">
         <is>
           <t>たけれ</t>
         </is>
       </c>
-      <c r="S16" s="21" t="inlineStr">
+      <c r="S16" s="20" t="inlineStr">
         <is>
           <t>まほしけれ</t>
         </is>
       </c>
-      <c r="T16" s="21" t="inlineStr">
+      <c r="T16" s="19" t="inlineStr">
         <is>
           <t>たれ</t>
         </is>
       </c>
-      <c r="U16" s="21" t="inlineStr">
+      <c r="U16" s="19" t="inlineStr">
         <is>
           <t>れ</t>
         </is>
       </c>
-      <c r="V16" s="21" t="inlineStr">
+      <c r="V16" s="19" t="inlineStr">
         <is>
           <t>つれ</t>
         </is>
       </c>
-      <c r="W16" s="21" t="inlineStr">
+      <c r="W16" s="19" t="inlineStr">
         <is>
           <t>ぬれ</t>
         </is>
       </c>
-      <c r="X16" s="21" t="inlineStr">
+      <c r="X16" s="19" t="inlineStr">
         <is>
           <t>けれ</t>
         </is>
       </c>
-      <c r="Y16" s="21" t="inlineStr">
+      <c r="Y16" s="19" t="inlineStr">
         <is>
           <t>しか</t>
         </is>
       </c>
-      <c r="Z16" s="21" t="inlineStr">
+      <c r="Z16" s="19" t="inlineStr">
         <is>
           <t>じ</t>
         </is>
       </c>
-      <c r="AA16" s="21" t="inlineStr">
+      <c r="AA16" s="19" t="inlineStr">
         <is>
           <t>ね
 ざれ</t>
         </is>
       </c>
-      <c r="AB16" s="22" t="inlineStr">
+      <c r="AB16" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="43" customHeight="1" thickBot="1">
-      <c r="A17" s="12" t="inlineStr">
+    <row r="17" ht="51" customHeight="1" thickBot="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>命令形</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>せよ</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>させよ</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>しめよ</t>
         </is>
       </c>
-      <c r="E17" s="23" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr">
         <is>
           <t>れよ</t>
         </is>
       </c>
-      <c r="F17" s="23" t="inlineStr">
+      <c r="F17" s="22" t="inlineStr">
         <is>
           <t>られよ</t>
         </is>
       </c>
-      <c r="G17" s="23" t="inlineStr">
+      <c r="G17" s="22" t="inlineStr">
         <is>
           <t>たまへ</t>
         </is>
       </c>
-      <c r="H17" s="23" t="inlineStr">
+      <c r="H17" s="22" t="inlineStr">
         <is>
           <t>なれ</t>
         </is>
       </c>
-      <c r="I17" s="23" t="inlineStr">
+      <c r="I17" s="22" t="inlineStr">
         <is>
           <t>たれ</t>
         </is>
       </c>
-      <c r="J17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T17" s="22" t="inlineStr">
         <is>
           <t>たれ</t>
         </is>
       </c>
-      <c r="U17" s="23" t="inlineStr">
+      <c r="U17" s="22" t="inlineStr">
         <is>
           <t>れ</t>
         </is>
       </c>
-      <c r="V17" s="23" t="inlineStr">
+      <c r="V17" s="22" t="inlineStr">
         <is>
           <t>てよ</t>
         </is>
       </c>
-      <c r="W17" s="23" t="inlineStr">
+      <c r="W17" s="22" t="inlineStr">
         <is>
           <t>ね</t>
         </is>
       </c>
-      <c r="X17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA17" s="23" t="inlineStr">
+      <c r="X17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z17" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA17" s="22" t="inlineStr">
         <is>
           <t>ざれ</t>
         </is>
       </c>
-      <c r="AB17" s="24" t="inlineStr">
+      <c r="AB17" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3212,15 +3223,15 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="V1:W1"/>
     <mergeCell ref="T1:U1"/>
     <mergeCell ref="H1:I1"/>
-    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="E1:F1"/>
     <mergeCell ref="L1:M1"/>
     <mergeCell ref="R1:S1"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.05" right="0.05" top="0.08" bottom="0.08" header="0" footer="0"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="64"/>
+  <pageMargins left="0.12" right="0.12" top="0.12" bottom="0.12" header="0.05" footer="0.05"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="68" fitToHeight="1" fitToWidth="1" pageOrder="overThenDown"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update study workbook templates
</commit_message>
<xml_diff>
--- a/Studymaterials/日本語助動詞一覧.xlsx
+++ b/Studymaterials/日本語助動詞一覧.xlsx
@@ -6,11 +6,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用言活用対応表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Sheet1'!$1:$1,'Sheet1'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1'!$A$1:$AB$17</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'用言活用対応表'!$1:$3,'用言活用対応表'!$A:$A</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'用言活用対応表'!$A$1:$N$21</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Sheet1'!$1:$1,'Sheet1'!$A:$A</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Sheet1'!$A$1:$AB$17</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
@@ -57,23 +60,42 @@
       <sz val="7"/>
     </font>
     <font>
-      <name val="Noto Sans JP"/>
+      <name val="Yu Gothic"/>
       <charset val="128"/>
       <family val="3"/>
       <b val="1"/>
-      <color rgb="FF000000"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="游ゴシック"/>
+      <name val="Yu Gothic"/>
       <charset val="128"/>
       <family val="3"/>
       <b val="1"/>
-      <color rgb="FF000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <i val="1"/>
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -100,8 +122,33 @@
         <fgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F7F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="17">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -314,6 +361,80 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -337,7 +458,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
@@ -411,11 +532,40 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -781,6 +931,1521 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13"/>
+  <cols>
+    <col width="7.1796875" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="8"/>
+    <col width="7.1796875" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="12"/>
+    <col width="7.1796875" customWidth="1" min="13" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>品詞</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
+        <is>
+          <t>動詞</t>
+        </is>
+      </c>
+      <c r="C1" s="33" t="n"/>
+      <c r="D1" s="33" t="n"/>
+      <c r="E1" s="33" t="n"/>
+      <c r="F1" s="33" t="n"/>
+      <c r="G1" s="33" t="n"/>
+      <c r="H1" s="33" t="n"/>
+      <c r="I1" s="33" t="n"/>
+      <c r="J1" s="32" t="n"/>
+      <c r="K1" s="31" t="inlineStr">
+        <is>
+          <t>形容詞</t>
+        </is>
+      </c>
+      <c r="L1" s="32" t="n"/>
+      <c r="M1" s="31" t="inlineStr">
+        <is>
+          <t>形容動詞</t>
+        </is>
+      </c>
+      <c r="N1" s="32" t="n"/>
+    </row>
+    <row r="2" ht="64" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>文語の
+活用</t>
+        </is>
+      </c>
+      <c r="B2" s="34" t="inlineStr">
+        <is>
+          <t>四段</t>
+        </is>
+      </c>
+      <c r="C2" s="34" t="inlineStr">
+        <is>
+          <t>上一段</t>
+        </is>
+      </c>
+      <c r="D2" s="34" t="inlineStr">
+        <is>
+          <t>上二段</t>
+        </is>
+      </c>
+      <c r="E2" s="34" t="inlineStr">
+        <is>
+          <t>下一段</t>
+        </is>
+      </c>
+      <c r="F2" s="34" t="inlineStr">
+        <is>
+          <t>下二段</t>
+        </is>
+      </c>
+      <c r="G2" s="34" t="inlineStr">
+        <is>
+          <t>ラ変</t>
+        </is>
+      </c>
+      <c r="H2" s="34" t="inlineStr">
+        <is>
+          <t>ナ変</t>
+        </is>
+      </c>
+      <c r="I2" s="34" t="inlineStr">
+        <is>
+          <t>サ変</t>
+        </is>
+      </c>
+      <c r="J2" s="34" t="inlineStr">
+        <is>
+          <t>カ変</t>
+        </is>
+      </c>
+      <c r="K2" s="34" t="inlineStr">
+        <is>
+          <t>ク</t>
+        </is>
+      </c>
+      <c r="L2" s="34" t="inlineStr">
+        <is>
+          <t>シク</t>
+        </is>
+      </c>
+      <c r="M2" s="34" t="inlineStr">
+        <is>
+          <t>ナリ</t>
+        </is>
+      </c>
+      <c r="N2" s="34" t="inlineStr">
+        <is>
+          <t>タリ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="82" customHeight="1">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>用言（文語）</t>
+        </is>
+      </c>
+      <c r="B3" s="34" t="inlineStr">
+        <is>
+          <t>書く</t>
+        </is>
+      </c>
+      <c r="C3" s="34" t="inlineStr">
+        <is>
+          <t>見る</t>
+        </is>
+      </c>
+      <c r="D3" s="34" t="inlineStr">
+        <is>
+          <t>起く</t>
+        </is>
+      </c>
+      <c r="E3" s="34" t="inlineStr">
+        <is>
+          <t>蹴る</t>
+        </is>
+      </c>
+      <c r="F3" s="34" t="inlineStr">
+        <is>
+          <t>受く</t>
+        </is>
+      </c>
+      <c r="G3" s="34" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="H3" s="34" t="inlineStr">
+        <is>
+          <t>死ぬ</t>
+        </is>
+      </c>
+      <c r="I3" s="34" t="inlineStr">
+        <is>
+          <t>す</t>
+        </is>
+      </c>
+      <c r="J3" s="34" t="inlineStr">
+        <is>
+          <t>来</t>
+        </is>
+      </c>
+      <c r="K3" s="34" t="inlineStr">
+        <is>
+          <t>高し</t>
+        </is>
+      </c>
+      <c r="L3" s="34" t="inlineStr">
+        <is>
+          <t>美し</t>
+        </is>
+      </c>
+      <c r="M3" s="34" t="inlineStr">
+        <is>
+          <t>静かなり</t>
+        </is>
+      </c>
+      <c r="N3" s="34" t="inlineStr">
+        <is>
+          <t>堂々たり</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>語幹（文語）</t>
+        </is>
+      </c>
+      <c r="B4" s="34" t="inlineStr">
+        <is>
+          <t>書</t>
+        </is>
+      </c>
+      <c r="C4" s="34" t="inlineStr">
+        <is>
+          <t>見</t>
+        </is>
+      </c>
+      <c r="D4" s="34" t="inlineStr">
+        <is>
+          <t>起</t>
+        </is>
+      </c>
+      <c r="E4" s="34" t="inlineStr">
+        <is>
+          <t>蹴</t>
+        </is>
+      </c>
+      <c r="F4" s="34" t="inlineStr">
+        <is>
+          <t>受</t>
+        </is>
+      </c>
+      <c r="G4" s="34" t="inlineStr">
+        <is>
+          <t>あ</t>
+        </is>
+      </c>
+      <c r="H4" s="34" t="inlineStr">
+        <is>
+          <t>死</t>
+        </is>
+      </c>
+      <c r="I4" s="34" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="J4" s="34" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="K4" s="34" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="L4" s="34" t="inlineStr">
+        <is>
+          <t>美し</t>
+        </is>
+      </c>
+      <c r="M4" s="34" t="inlineStr">
+        <is>
+          <t>静か</t>
+        </is>
+      </c>
+      <c r="N4" s="34" t="inlineStr">
+        <is>
+          <t>堂々</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+未然形</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>か</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>き</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>け</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>ら</t>
+        </is>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>な</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="inlineStr">
+        <is>
+          <t>せ</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="inlineStr">
+        <is>
+          <t>こ</t>
+        </is>
+      </c>
+      <c r="K5" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="L5" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="M5" s="28" t="inlineStr">
+        <is>
+          <t>なら</t>
+        </is>
+      </c>
+      <c r="N5" s="28" t="inlineStr">
+        <is>
+          <t>たら</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+連用形</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>き</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>き</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>け</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>り</t>
+        </is>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>に</t>
+        </is>
+      </c>
+      <c r="I6" s="28" t="inlineStr">
+        <is>
+          <t>し</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>き</t>
+        </is>
+      </c>
+      <c r="K6" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="L6" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="M6" s="28" t="inlineStr">
+        <is>
+          <t>なり
+に</t>
+        </is>
+      </c>
+      <c r="N6" s="28" t="inlineStr">
+        <is>
+          <t>たり
+と</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+終止形</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>り</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>ぬ</t>
+        </is>
+      </c>
+      <c r="I7" s="28" t="inlineStr">
+        <is>
+          <t>す</t>
+        </is>
+      </c>
+      <c r="J7" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>し</t>
+        </is>
+      </c>
+      <c r="L7" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="M7" s="28" t="inlineStr">
+        <is>
+          <t>なり</t>
+        </is>
+      </c>
+      <c r="N7" s="28" t="inlineStr">
+        <is>
+          <t>たり</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+連体形</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>くる</t>
+        </is>
+      </c>
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>くる</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="H8" s="28" t="inlineStr">
+        <is>
+          <t>ぬる</t>
+        </is>
+      </c>
+      <c r="I8" s="28" t="inlineStr">
+        <is>
+          <t>する</t>
+        </is>
+      </c>
+      <c r="J8" s="28" t="inlineStr">
+        <is>
+          <t>くる</t>
+        </is>
+      </c>
+      <c r="K8" s="28" t="inlineStr">
+        <is>
+          <t>き</t>
+        </is>
+      </c>
+      <c r="L8" s="28" t="inlineStr">
+        <is>
+          <t>き</t>
+        </is>
+      </c>
+      <c r="M8" s="28" t="inlineStr">
+        <is>
+          <t>なる</t>
+        </is>
+      </c>
+      <c r="N8" s="28" t="inlineStr">
+        <is>
+          <t>たる</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+已然形</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>け</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>くれ</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>くれ</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="H9" s="28" t="inlineStr">
+        <is>
+          <t>ぬれ</t>
+        </is>
+      </c>
+      <c r="I9" s="28" t="inlineStr">
+        <is>
+          <t>すれ</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="inlineStr">
+        <is>
+          <t>くれ</t>
+        </is>
+      </c>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>けれ</t>
+        </is>
+      </c>
+      <c r="L9" s="28" t="inlineStr">
+        <is>
+          <t>けれ</t>
+        </is>
+      </c>
+      <c r="M9" s="28" t="inlineStr">
+        <is>
+          <t>なれ</t>
+        </is>
+      </c>
+      <c r="N9" s="28" t="inlineStr">
+        <is>
+          <t>たれ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+命令形</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>け</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>よ</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>きよ</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>よ</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>けよ</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>ね</t>
+        </is>
+      </c>
+      <c r="I10" s="28" t="inlineStr">
+        <is>
+          <t>せよ</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="inlineStr">
+        <is>
+          <t>こ
+こよ</t>
+        </is>
+      </c>
+      <c r="K10" s="28" t="n"/>
+      <c r="L10" s="28" t="n"/>
+      <c r="M10" s="28" t="inlineStr">
+        <is>
+          <t>なれ</t>
+        </is>
+      </c>
+      <c r="N10" s="28" t="inlineStr">
+        <is>
+          <t>たれ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="204" customHeight="1">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>対応メモ
+（文語）</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>文語の基本的な動詞活用</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>例: 見る
+射る
+着る
+覚え方:
+ひいきにみゐる</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>二段活用。終止・連体で母音が変わる</t>
+        </is>
+      </c>
+      <c r="E11" s="30" t="inlineStr">
+        <is>
+          <t>文語では例が少ない</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>二段活用。終止・連体で母音が変わる</t>
+        </is>
+      </c>
+      <c r="G11" s="30" t="inlineStr">
+        <is>
+          <t>あり・をり・はべり・いまそかり</t>
+        </is>
+      </c>
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>死ぬ・往ぬ</t>
+        </is>
+      </c>
+      <c r="I11" s="30" t="inlineStr">
+        <is>
+          <t>す・おはす</t>
+        </is>
+      </c>
+      <c r="J11" s="30" t="inlineStr">
+        <is>
+          <t>来のみ</t>
+        </is>
+      </c>
+      <c r="K11" s="30" t="inlineStr">
+        <is>
+          <t>形容詞ク活用</t>
+        </is>
+      </c>
+      <c r="L11" s="30" t="inlineStr">
+        <is>
+          <t>形容詞シク活用</t>
+        </is>
+      </c>
+      <c r="M11" s="30" t="inlineStr">
+        <is>
+          <t>形容動詞ナリ活用</t>
+        </is>
+      </c>
+      <c r="N11" s="30" t="inlineStr">
+        <is>
+          <t>形容動詞タリ活用</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="82" customHeight="1">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>用言（口語）</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="inlineStr">
+        <is>
+          <t>書く</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>見る</t>
+        </is>
+      </c>
+      <c r="D12" s="34" t="inlineStr">
+        <is>
+          <t>起きる</t>
+        </is>
+      </c>
+      <c r="E12" s="34" t="inlineStr">
+        <is>
+          <t>蹴る</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>受ける</t>
+        </is>
+      </c>
+      <c r="G12" s="34" t="inlineStr">
+        <is>
+          <t>ある</t>
+        </is>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>死ぬ</t>
+        </is>
+      </c>
+      <c r="I12" s="34" t="inlineStr">
+        <is>
+          <t>する</t>
+        </is>
+      </c>
+      <c r="J12" s="34" t="inlineStr">
+        <is>
+          <t>来る</t>
+        </is>
+      </c>
+      <c r="K12" s="34" t="inlineStr">
+        <is>
+          <t>高い</t>
+        </is>
+      </c>
+      <c r="L12" s="34" t="inlineStr">
+        <is>
+          <t>美しい</t>
+        </is>
+      </c>
+      <c r="M12" s="34" t="inlineStr">
+        <is>
+          <t>静かだ</t>
+        </is>
+      </c>
+      <c r="N12" s="38" t="inlineStr">
+        <is>
+          <t>堂々と
+している</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>口語の活用</t>
+        </is>
+      </c>
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>五段</t>
+        </is>
+      </c>
+      <c r="C13" s="34" t="inlineStr">
+        <is>
+          <t>上一段</t>
+        </is>
+      </c>
+      <c r="D13" s="34" t="inlineStr">
+        <is>
+          <t>上一段</t>
+        </is>
+      </c>
+      <c r="E13" s="34" t="inlineStr">
+        <is>
+          <t>五段</t>
+        </is>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>下一段</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>五段</t>
+        </is>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>五段</t>
+        </is>
+      </c>
+      <c r="I13" s="34" t="inlineStr">
+        <is>
+          <t>サ変</t>
+        </is>
+      </c>
+      <c r="J13" s="34" t="inlineStr">
+        <is>
+          <t>カ変</t>
+        </is>
+      </c>
+      <c r="K13" s="34" t="inlineStr">
+        <is>
+          <t>形容詞</t>
+        </is>
+      </c>
+      <c r="L13" s="32" t="n"/>
+      <c r="M13" s="34" t="inlineStr">
+        <is>
+          <t>形容動詞</t>
+        </is>
+      </c>
+      <c r="N13" s="32" t="n"/>
+    </row>
+    <row r="14" ht="86" customHeight="1">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>語幹（口語）</t>
+        </is>
+      </c>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>書</t>
+        </is>
+      </c>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>見</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>起き</t>
+        </is>
+      </c>
+      <c r="E14" s="34" t="inlineStr">
+        <is>
+          <t>蹴</t>
+        </is>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>受け</t>
+        </is>
+      </c>
+      <c r="G14" s="34" t="inlineStr">
+        <is>
+          <t>あ</t>
+        </is>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>死</t>
+        </is>
+      </c>
+      <c r="I14" s="34" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="J14" s="34" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="K14" s="34" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="L14" s="34" t="inlineStr">
+        <is>
+          <t>美し</t>
+        </is>
+      </c>
+      <c r="M14" s="34" t="inlineStr">
+        <is>
+          <t>静か</t>
+        </is>
+      </c>
+      <c r="N14" s="34" t="inlineStr">
+        <is>
+          <t>堂々</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+未然形</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>か
+こ</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>ら
+ろ</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="inlineStr">
+        <is>
+          <t>ら
+ろ</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="inlineStr">
+        <is>
+          <t>な
+の</t>
+        </is>
+      </c>
+      <c r="I15" s="28" t="inlineStr">
+        <is>
+          <t>し
+せ
+さ</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="inlineStr">
+        <is>
+          <t>こ</t>
+        </is>
+      </c>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>かろ</t>
+        </is>
+      </c>
+      <c r="L15" s="28" t="inlineStr">
+        <is>
+          <t>かろ</t>
+        </is>
+      </c>
+      <c r="M15" s="28" t="inlineStr">
+        <is>
+          <t>だろ</t>
+        </is>
+      </c>
+      <c r="N15" s="28" t="inlineStr">
+        <is>
+          <t>としてい</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+連用形</t>
+        </is>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>き
+い</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>り
+っ</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>り
+っ</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="inlineStr">
+        <is>
+          <t>に
+ん</t>
+        </is>
+      </c>
+      <c r="I16" s="28" t="inlineStr">
+        <is>
+          <t>し</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="inlineStr">
+        <is>
+          <t>き</t>
+        </is>
+      </c>
+      <c r="K16" s="28" t="inlineStr">
+        <is>
+          <t>く
+かっ</t>
+        </is>
+      </c>
+      <c r="L16" s="28" t="inlineStr">
+        <is>
+          <t>く
+かっ</t>
+        </is>
+      </c>
+      <c r="M16" s="28" t="inlineStr">
+        <is>
+          <t>で
+に
+だっ</t>
+        </is>
+      </c>
+      <c r="N16" s="28" t="inlineStr">
+        <is>
+          <t>として</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+終止形</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="F17" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="H17" s="28" t="inlineStr">
+        <is>
+          <t>ぬ</t>
+        </is>
+      </c>
+      <c r="I17" s="28" t="inlineStr">
+        <is>
+          <t>する</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="inlineStr">
+        <is>
+          <t>くる</t>
+        </is>
+      </c>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>い</t>
+        </is>
+      </c>
+      <c r="L17" s="28" t="inlineStr">
+        <is>
+          <t>い</t>
+        </is>
+      </c>
+      <c r="M17" s="28" t="inlineStr">
+        <is>
+          <t>だ</t>
+        </is>
+      </c>
+      <c r="N17" s="28" t="inlineStr">
+        <is>
+          <t>としている</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+連体形</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>く</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="E18" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="inlineStr">
+        <is>
+          <t>る</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="inlineStr">
+        <is>
+          <t>ぬ</t>
+        </is>
+      </c>
+      <c r="I18" s="28" t="inlineStr">
+        <is>
+          <t>する</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="inlineStr">
+        <is>
+          <t>くる</t>
+        </is>
+      </c>
+      <c r="K18" s="28" t="inlineStr">
+        <is>
+          <t>い</t>
+        </is>
+      </c>
+      <c r="L18" s="28" t="inlineStr">
+        <is>
+          <t>い</t>
+        </is>
+      </c>
+      <c r="M18" s="28" t="inlineStr">
+        <is>
+          <t>な</t>
+        </is>
+      </c>
+      <c r="N18" s="28" t="inlineStr">
+        <is>
+          <t>とした</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+仮定形</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>け</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="E19" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="F19" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="H19" s="28" t="inlineStr">
+        <is>
+          <t>ね</t>
+        </is>
+      </c>
+      <c r="I19" s="28" t="inlineStr">
+        <is>
+          <t>すれ</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="inlineStr">
+        <is>
+          <t>くれ</t>
+        </is>
+      </c>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>けれ</t>
+        </is>
+      </c>
+      <c r="L19" s="28" t="inlineStr">
+        <is>
+          <t>けれ</t>
+        </is>
+      </c>
+      <c r="M19" s="28" t="inlineStr">
+        <is>
+          <t>なら</t>
+        </is>
+      </c>
+      <c r="N19" s="28" t="inlineStr">
+        <is>
+          <t>としていれ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>語尾
+命令形</t>
+        </is>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>け</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="inlineStr">
+        <is>
+          <t>ろ
+よ</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
+        <is>
+          <t>ろ
+よ</t>
+        </is>
+      </c>
+      <c r="E20" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="F20" s="28" t="inlineStr">
+        <is>
+          <t>ろ
+よ</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="inlineStr">
+        <is>
+          <t>れ</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="inlineStr">
+        <is>
+          <t>ね</t>
+        </is>
+      </c>
+      <c r="I20" s="28" t="inlineStr">
+        <is>
+          <t>しろ
+せよ</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="inlineStr">
+        <is>
+          <t>こい</t>
+        </is>
+      </c>
+      <c r="K20" s="28" t="n"/>
+      <c r="L20" s="28" t="n"/>
+      <c r="M20" s="28" t="n"/>
+      <c r="N20" s="28" t="inlineStr">
+        <is>
+          <t>としていろ</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="204" customHeight="1">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>対応メモ
+（口語）</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では多くが五段に対応</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>現代語でも上一段に対応</t>
+        </is>
+      </c>
+      <c r="D21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では上一段に合流</t>
+        </is>
+      </c>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では五段に対応する例として扱う</t>
+        </is>
+      </c>
+      <c r="F21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では下一段に合流</t>
+        </is>
+      </c>
+      <c r="G21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では五段に合流</t>
+        </is>
+      </c>
+      <c r="H21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では五段に合流</t>
+        </is>
+      </c>
+      <c r="I21" s="30" t="inlineStr">
+        <is>
+          <t>現代語でもサ変</t>
+        </is>
+      </c>
+      <c r="J21" s="30" t="inlineStr">
+        <is>
+          <t>現代語でもカ変</t>
+        </is>
+      </c>
+      <c r="K21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では形容詞</t>
+        </is>
+      </c>
+      <c r="L21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では形容詞</t>
+        </is>
+      </c>
+      <c r="M21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では形容動詞</t>
+        </is>
+      </c>
+      <c r="N21" s="30" t="inlineStr">
+        <is>
+          <t>現代語では形容動詞相当として扱う</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="M13:N13"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.42" right="0.42" top="0.55" bottom="0.55" header="0.08" footer="0.08"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="53"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13"/>
   <cols>
@@ -788,8 +2453,9 @@
     <col width="4.6328125" customWidth="1" min="2" max="6"/>
     <col width="7.453125" customWidth="1" min="7" max="8"/>
     <col width="5.6328125" customWidth="1" min="9" max="9"/>
-    <col width="4.6328125" customWidth="1" min="10" max="13"/>
-    <col width="5.6328125" customWidth="1" min="14" max="15"/>
+    <col width="4.6328125" customWidth="1" min="10" max="12"/>
+    <col width="7.1796875" customWidth="1" min="13" max="14"/>
+    <col width="5.6328125" customWidth="1" min="15" max="15"/>
     <col width="4.6328125" customWidth="1" min="16" max="17"/>
     <col width="5.6328125" customWidth="1" min="18" max="19"/>
     <col width="4.6328125" customWidth="1" min="20" max="20"/>
@@ -807,14 +2473,14 @@
           <t>分類</t>
         </is>
       </c>
-      <c r="B1" s="25" t="inlineStr">
+      <c r="B1" s="35" t="inlineStr">
         <is>
           <t>使役</t>
         </is>
       </c>
-      <c r="C1" s="26" t="n"/>
-      <c r="D1" s="27" t="n"/>
-      <c r="E1" s="25" t="inlineStr">
+      <c r="C1" s="36" t="n"/>
+      <c r="D1" s="37" t="n"/>
+      <c r="E1" s="35" t="inlineStr">
         <is>
           <t>受身
 尊敬
@@ -822,91 +2488,91 @@
 自発</t>
         </is>
       </c>
-      <c r="F1" s="27" t="n"/>
-      <c r="G1" s="25" t="inlineStr">
+      <c r="F1" s="37" t="n"/>
+      <c r="G1" s="35" t="inlineStr">
         <is>
           <t>尊敬</t>
         </is>
       </c>
-      <c r="H1" s="25" t="inlineStr">
+      <c r="H1" s="35" t="inlineStr">
         <is>
           <t>断定</t>
         </is>
       </c>
-      <c r="I1" s="27" t="n"/>
-      <c r="J1" s="25" t="inlineStr">
+      <c r="I1" s="37" t="n"/>
+      <c r="J1" s="35" t="inlineStr">
         <is>
           <t>比況</t>
         </is>
       </c>
-      <c r="K1" s="25" t="inlineStr">
+      <c r="K1" s="35" t="inlineStr">
         <is>
           <t>伝聞</t>
         </is>
       </c>
-      <c r="L1" s="25" t="inlineStr">
+      <c r="L1" s="35" t="inlineStr">
         <is>
           <t>推定</t>
         </is>
       </c>
-      <c r="M1" s="27" t="n"/>
-      <c r="N1" s="25" t="inlineStr">
+      <c r="M1" s="37" t="n"/>
+      <c r="N1" s="35" t="inlineStr">
         <is>
           <t>当然
 推量</t>
         </is>
       </c>
-      <c r="O1" s="25" t="inlineStr">
+      <c r="O1" s="35" t="inlineStr">
         <is>
           <t>意志
 推量</t>
         </is>
       </c>
-      <c r="P1" s="25" t="inlineStr">
+      <c r="P1" s="35" t="inlineStr">
         <is>
           <t>現在推量</t>
         </is>
       </c>
-      <c r="Q1" s="25" t="inlineStr">
+      <c r="Q1" s="35" t="inlineStr">
         <is>
           <t>過去推量</t>
         </is>
       </c>
-      <c r="R1" s="25" t="inlineStr">
+      <c r="R1" s="35" t="inlineStr">
         <is>
           <t>希望</t>
         </is>
       </c>
-      <c r="S1" s="27" t="n"/>
-      <c r="T1" s="25" t="inlineStr">
+      <c r="S1" s="37" t="n"/>
+      <c r="T1" s="35" t="inlineStr">
         <is>
           <t>存続</t>
         </is>
       </c>
-      <c r="U1" s="27" t="n"/>
-      <c r="V1" s="25" t="inlineStr">
+      <c r="U1" s="37" t="n"/>
+      <c r="V1" s="35" t="inlineStr">
         <is>
           <t>完了</t>
         </is>
       </c>
-      <c r="W1" s="27" t="n"/>
-      <c r="X1" s="25" t="inlineStr">
+      <c r="W1" s="37" t="n"/>
+      <c r="X1" s="35" t="inlineStr">
         <is>
           <t>過去
 詠嘆</t>
         </is>
       </c>
-      <c r="Y1" s="25" t="inlineStr">
+      <c r="Y1" s="35" t="inlineStr">
         <is>
           <t>過去</t>
         </is>
       </c>
-      <c r="Z1" s="25" t="inlineStr">
+      <c r="Z1" s="35" t="inlineStr">
         <is>
           <t>打消推量</t>
         </is>
       </c>
-      <c r="AA1" s="25" t="inlineStr">
+      <c r="AA1" s="35" t="inlineStr">
         <is>
           <t>打消</t>
         </is>
@@ -920,7 +2586,8 @@
     <row r="2" ht="76" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>現代口語</t>
+          <t>文語の
+活用</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1064,7 +2731,8 @@
     <row r="3" ht="51" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>接続</t>
+          <t>用言
+（文語）</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1208,7 +2876,8 @@
     <row r="4" ht="61" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>未然形</t>
+          <t>語幹
+（文語）</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2424,8 +4093,8 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>べく
-べから</t>
+          <t>堂々と
+している</t>
         </is>
       </c>
       <c r="O12" s="19" t="inlineStr">
@@ -2504,7 +4173,8 @@
     <row r="13" ht="81" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>連用形</t>
+          <t>語幹
+（口語）</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
@@ -3232,6 +4902,6 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.12" right="0.12" top="0.12" bottom="0.12" header="0.05" footer="0.05"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="68" fitToHeight="1" fitToWidth="1" pageOrder="overThenDown"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="66" pageOrder="overThenDown"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Japanese auxiliary verbs workbook
</commit_message>
<xml_diff>
--- a/Studymaterials/日本語助動詞一覧.xlsx
+++ b/Studymaterials/日本語助動詞一覧.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakag\Desktop\GitHub\Myownproject\Studymaterials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23970728-F59C-4A56-AFA4-6A7DFA79D7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{906E9BDB-44AB-404A-834F-A574DCCA0E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Sheet1!$B$1:$AC$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">用言活用対応表!$B$1:$O$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">用言活用対応表!$B$1:$P$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">Sheet1!$1:$1,Sheet1!$B:$B</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">用言活用対応表!$A:$B,用言活用対応表!$1:$3</definedName>
   </definedNames>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="315">
   <si>
     <t>品詞</t>
   </si>
@@ -274,15 +274,6 @@
   </si>
   <si>
     <t>文語の基本的な動詞活用</t>
-  </si>
-  <si>
-    <t>二段活用。終止・連体で母音が変わる</t>
-  </si>
-  <si>
-    <t>文語では例が少ない</t>
-  </si>
-  <si>
-    <t>来のみ</t>
   </si>
   <si>
     <t>形容詞ク活用</t>
@@ -354,9 +345,6 @@
     <t>だろ</t>
   </si>
   <si>
-    <t>としてい</t>
-  </si>
-  <si>
     <t>き
 い</t>
   </si>
@@ -378,22 +366,10 @@
 だっ</t>
   </si>
   <si>
-    <t>として</t>
-  </si>
-  <si>
     <t>い</t>
   </si>
   <si>
     <t>だ</t>
-  </si>
-  <si>
-    <t>としている</t>
-  </si>
-  <si>
-    <t>とした</t>
-  </si>
-  <si>
-    <t>としていれ</t>
   </si>
   <si>
     <t>ろ
@@ -405,9 +381,6 @@
   </si>
   <si>
     <t>こい</t>
-  </si>
-  <si>
-    <t>としていろ</t>
   </si>
   <si>
     <t>対応メモ
@@ -1056,11 +1029,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>全体は連語。
-「する」はサ変</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>現代語でも形容詞</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -1072,6 +1040,159 @@
   <si>
     <t>あり/をり/
 はべり/いまそかり</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">九語とその
+複合動詞のみ </t>
+    <rPh sb="0" eb="2">
+      <t>キュウゴ</t>
+    </rPh>
+    <rPh sb="6" eb="10">
+      <t>フクゴウドウシ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「蹴る」のみ</t>
+    <rPh sb="1" eb="2">
+      <t>ケ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>終止・連体がウ段
+他の三つがイ段</t>
+    <rPh sb="0" eb="2">
+      <t>シュウシ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>レンタイ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>タ</t>
+    </rPh>
+    <rPh sb="11" eb="12">
+      <t>ミ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>ダン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>終止・連体がウ段
+他の三つがエ段</t>
+    <rPh sb="0" eb="2">
+      <t>シュウシ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>レンタイ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>タ</t>
+    </rPh>
+    <rPh sb="11" eb="12">
+      <t>ミ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>ダン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「来」のみ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>堂々としてい</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ろ
+よ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>上一段</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>補助動詞「いる」の
+上一段</t>
+    <rPh sb="0" eb="4">
+      <t>ホジョドウシ</t>
+    </rPh>
+    <rPh sb="10" eb="13">
+      <t>カミイチダン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>上一段の九語は「ひいきにみゐる」と覚える方法がある。
+「ひ」は「干る」、「い」は「射る」・「鋳る」、「き」は「着る」、「に」は「似る」・「煮る」、「み」は「見る」、「ゐ」は「居る」・「率る」。</t>
+    <rPh sb="17" eb="18">
+      <t>オボ</t>
+    </rPh>
+    <rPh sb="20" eb="22">
+      <t>ホウホウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「堂々たり」の現代口語訳は「堂々と」という副詞とも考えられる。
+ここでは、用言としての機能をも耐えるために「堂々としている」とした。これは副詞「堂々と」＋サ変動詞「し」の連用形＋助詞「で」＋補助動詞「いる」から構成される。</t>
+    <rPh sb="1" eb="3">
+      <t>ドウドウ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ゲンダイ</t>
+    </rPh>
+    <rPh sb="9" eb="12">
+      <t>コウゴヤク</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>ドウドウ</t>
+    </rPh>
+    <rPh sb="21" eb="23">
+      <t>フクシ</t>
+    </rPh>
+    <rPh sb="25" eb="26">
+      <t>カンガ</t>
+    </rPh>
+    <rPh sb="37" eb="39">
+      <t>ヨウゲン</t>
+    </rPh>
+    <rPh sb="43" eb="45">
+      <t>キノウ</t>
+    </rPh>
+    <rPh sb="47" eb="48">
+      <t>タ</t>
+    </rPh>
+    <rPh sb="54" eb="56">
+      <t>ドウドウ</t>
+    </rPh>
+    <rPh sb="69" eb="71">
+      <t>フクシ</t>
+    </rPh>
+    <rPh sb="72" eb="74">
+      <t>ドウドウ</t>
+    </rPh>
+    <rPh sb="78" eb="81">
+      <t>ヘンドウシ</t>
+    </rPh>
+    <rPh sb="85" eb="88">
+      <t>レンヨウケイ</t>
+    </rPh>
+    <rPh sb="89" eb="91">
+      <t>ジョシ</t>
+    </rPh>
+    <rPh sb="95" eb="99">
+      <t>ホジョドウシ</t>
+    </rPh>
+    <rPh sb="105" eb="107">
+      <t>コウセイ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1079,7 +1200,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1169,6 +1290,13 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -1223,7 +1351,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="46">
+  <borders count="47">
     <border>
       <left/>
       <right/>
@@ -1826,11 +1954,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
@@ -1910,121 +2047,130 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2332,7 +2478,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="13"/>
   <cols>
     <col min="1" max="9" width="6" customWidth="1"/>
@@ -2340,38 +2486,39 @@
     <col min="11" max="13" width="6" customWidth="1"/>
     <col min="14" max="14" width="8" customWidth="1"/>
     <col min="15" max="15" width="7.1796875" customWidth="1"/>
+    <col min="16" max="16" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="24" customHeight="1">
-      <c r="A1" s="50" t="s">
+    <row r="1" spans="1:16" ht="24" customHeight="1">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="52" t="s">
+      <c r="B1" s="56"/>
+      <c r="C1" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
-      <c r="I1" s="53"/>
-      <c r="J1" s="53"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="52" t="s">
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="54"/>
-      <c r="N1" s="52" t="s">
+      <c r="M1" s="50"/>
+      <c r="N1" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="58"/>
+      <c r="O1" s="52"/>
     </row>
-    <row r="2" spans="1:15" ht="64" customHeight="1">
-      <c r="A2" s="45" t="s">
+    <row r="2" spans="1:16" ht="64" customHeight="1">
+      <c r="A2" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="29"/>
+      <c r="B2" s="42"/>
       <c r="C2" s="24" t="s">
         <v>5</v>
       </c>
@@ -2408,15 +2555,18 @@
       <c r="N2" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="59" t="s">
+      <c r="O2" s="28" t="s">
         <v>17</v>
       </c>
+      <c r="P2" s="72" t="s">
+        <v>313</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" ht="82" customHeight="1">
-      <c r="A3" s="46" t="s">
-        <v>294</v>
-      </c>
-      <c r="B3" s="29"/>
+    <row r="3" spans="1:16" ht="82" customHeight="1">
+      <c r="A3" s="43" t="s">
+        <v>285</v>
+      </c>
+      <c r="B3" s="42"/>
       <c r="C3" s="24" t="s">
         <v>18</v>
       </c>
@@ -2453,15 +2603,16 @@
       <c r="N3" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="O3" s="59" t="s">
+      <c r="O3" s="28" t="s">
         <v>30</v>
       </c>
+      <c r="P3" s="72"/>
     </row>
-    <row r="4" spans="1:15" ht="78" customHeight="1">
-      <c r="A4" s="46" t="s">
-        <v>293</v>
-      </c>
-      <c r="B4" s="29"/>
+    <row r="4" spans="1:16" ht="78" customHeight="1">
+      <c r="A4" s="43" t="s">
+        <v>284</v>
+      </c>
+      <c r="B4" s="42"/>
       <c r="C4" s="24" t="s">
         <v>31</v>
       </c>
@@ -2498,16 +2649,17 @@
       <c r="N4" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="O4" s="59" t="s">
+      <c r="O4" s="28" t="s">
         <v>41</v>
       </c>
+      <c r="P4" s="72"/>
     </row>
-    <row r="5" spans="1:15" ht="48" customHeight="1">
-      <c r="A5" s="47" t="s">
-        <v>299</v>
+    <row r="5" spans="1:16" ht="48" customHeight="1">
+      <c r="A5" s="46" t="s">
+        <v>290</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="C5" s="25" t="s">
         <v>42</v>
@@ -2545,14 +2697,15 @@
       <c r="N5" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="O5" s="60" t="s">
+      <c r="O5" s="29" t="s">
         <v>52</v>
       </c>
+      <c r="P5" s="72"/>
     </row>
-    <row r="6" spans="1:15" ht="48" customHeight="1">
-      <c r="A6" s="48"/>
+    <row r="6" spans="1:16" ht="48" customHeight="1">
+      <c r="A6" s="47"/>
       <c r="B6" s="26" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C6" s="25" t="s">
         <v>44</v>
@@ -2590,14 +2743,15 @@
       <c r="N6" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="O6" s="60" t="s">
+      <c r="O6" s="29" t="s">
         <v>57</v>
       </c>
+      <c r="P6" s="72"/>
     </row>
-    <row r="7" spans="1:15" ht="48" customHeight="1">
-      <c r="A7" s="48"/>
+    <row r="7" spans="1:16" ht="48" customHeight="1">
+      <c r="A7" s="47"/>
       <c r="B7" s="26" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>50</v>
@@ -2635,14 +2789,15 @@
       <c r="N7" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="O7" s="60" t="s">
+      <c r="O7" s="29" t="s">
         <v>61</v>
       </c>
+      <c r="P7" s="72"/>
     </row>
-    <row r="8" spans="1:15" ht="48" customHeight="1">
-      <c r="A8" s="48"/>
+    <row r="8" spans="1:16" ht="48" customHeight="1">
+      <c r="A8" s="47"/>
       <c r="B8" s="26" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>50</v>
@@ -2680,14 +2835,15 @@
       <c r="N8" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="O8" s="60" t="s">
+      <c r="O8" s="29" t="s">
         <v>66</v>
       </c>
+      <c r="P8" s="72"/>
     </row>
-    <row r="9" spans="1:15" ht="48" customHeight="1">
-      <c r="A9" s="48"/>
+    <row r="9" spans="1:16" ht="48" customHeight="1">
+      <c r="A9" s="47"/>
       <c r="B9" s="26" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>45</v>
@@ -2725,148 +2881,154 @@
       <c r="N9" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="O9" s="60" t="s">
+      <c r="O9" s="29" t="s">
         <v>73</v>
       </c>
+      <c r="P9" s="72"/>
     </row>
-    <row r="10" spans="1:15" ht="48" customHeight="1">
-      <c r="A10" s="48"/>
-      <c r="B10" s="67" t="s">
+    <row r="10" spans="1:16" ht="48" customHeight="1">
+      <c r="A10" s="47"/>
+      <c r="B10" s="33" t="s">
+        <v>282</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="J10" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="K10" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="O10" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="P10" s="72"/>
+    </row>
+    <row r="11" spans="1:16" ht="147" customHeight="1" thickBot="1">
+      <c r="A11" s="39" t="s">
+        <v>286</v>
+      </c>
+      <c r="B11" s="40"/>
+      <c r="C11" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>306</v>
+      </c>
+      <c r="F11" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="G11" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="H11" s="27" t="s">
+        <v>303</v>
+      </c>
+      <c r="I11" s="27" t="s">
         <v>291</v>
       </c>
-      <c r="C10" s="68" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="68" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" s="68" t="s">
-        <v>75</v>
-      </c>
-      <c r="F10" s="68" t="s">
-        <v>74</v>
-      </c>
-      <c r="G10" s="68" t="s">
-        <v>76</v>
-      </c>
-      <c r="H10" s="68" t="s">
-        <v>67</v>
-      </c>
-      <c r="I10" s="68" t="s">
-        <v>77</v>
-      </c>
-      <c r="J10" s="68" t="s">
-        <v>78</v>
-      </c>
-      <c r="K10" s="68" t="s">
-        <v>79</v>
-      </c>
-      <c r="L10" s="68"/>
-      <c r="M10" s="68"/>
-      <c r="N10" s="68" t="s">
-        <v>72</v>
-      </c>
-      <c r="O10" s="69" t="s">
-        <v>73</v>
-      </c>
+      <c r="J11" s="27" t="s">
+        <v>292</v>
+      </c>
+      <c r="K11" s="27" t="s">
+        <v>308</v>
+      </c>
+      <c r="L11" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="M11" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="N11" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="O11" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="P11" s="72"/>
     </row>
-    <row r="11" spans="1:15" ht="147" customHeight="1" thickBot="1">
-      <c r="A11" s="55" t="s">
-        <v>295</v>
-      </c>
-      <c r="B11" s="56"/>
-      <c r="C11" s="57" t="s">
-        <v>80</v>
-      </c>
-      <c r="D11" s="57" t="s">
-        <v>285</v>
-      </c>
-      <c r="E11" s="57" t="s">
-        <v>81</v>
-      </c>
-      <c r="F11" s="57" t="s">
-        <v>82</v>
-      </c>
-      <c r="G11" s="57" t="s">
-        <v>81</v>
-      </c>
-      <c r="H11" s="57" t="s">
-        <v>313</v>
-      </c>
-      <c r="I11" s="57" t="s">
-        <v>300</v>
-      </c>
-      <c r="J11" s="57" t="s">
-        <v>301</v>
-      </c>
-      <c r="K11" s="57" t="s">
-        <v>83</v>
-      </c>
-      <c r="L11" s="57" t="s">
-        <v>84</v>
-      </c>
-      <c r="M11" s="57" t="s">
+    <row r="12" spans="1:16" ht="82" customHeight="1">
+      <c r="A12" s="44" t="s">
+        <v>287</v>
+      </c>
+      <c r="B12" s="45"/>
+      <c r="C12" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="32" t="s">
         <v>85</v>
       </c>
-      <c r="N11" s="57" t="s">
+      <c r="F12" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="32" t="s">
         <v>86</v>
       </c>
-      <c r="O11" s="63" t="s">
+      <c r="H12" s="32" t="s">
         <v>87</v>
       </c>
+      <c r="I12" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="K12" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="L12" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="M12" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="N12" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="O12" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="P12" s="72" t="s">
+        <v>314</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" ht="82" customHeight="1">
-      <c r="A12" s="64" t="s">
-        <v>296</v>
-      </c>
-      <c r="B12" s="65"/>
-      <c r="C12" s="66" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="66" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="66" t="s">
-        <v>88</v>
-      </c>
-      <c r="F12" s="66" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="66" t="s">
-        <v>89</v>
-      </c>
-      <c r="H12" s="66" t="s">
-        <v>90</v>
-      </c>
-      <c r="I12" s="66" t="s">
-        <v>24</v>
-      </c>
-      <c r="J12" s="66" t="s">
-        <v>64</v>
-      </c>
-      <c r="K12" s="66" t="s">
-        <v>91</v>
-      </c>
-      <c r="L12" s="66" t="s">
-        <v>92</v>
-      </c>
-      <c r="M12" s="66" t="s">
+    <row r="13" spans="1:16" ht="70" customHeight="1">
+      <c r="A13" s="43" t="s">
+        <v>288</v>
+      </c>
+      <c r="B13" s="42"/>
+      <c r="C13" s="24" t="s">
         <v>93</v>
-      </c>
-      <c r="N12" s="66" t="s">
-        <v>94</v>
-      </c>
-      <c r="O12" s="61" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" ht="70" customHeight="1">
-      <c r="A13" s="46" t="s">
-        <v>297</v>
-      </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="24" t="s">
-        <v>96</v>
       </c>
       <c r="D13" s="24" t="s">
         <v>6</v>
@@ -2875,16 +3037,16 @@
         <v>6</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G13" s="24" t="s">
         <v>8</v>
       </c>
       <c r="H13" s="24" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I13" s="24" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="J13" s="24" t="s">
         <v>12</v>
@@ -2892,22 +3054,23 @@
       <c r="K13" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="L13" s="28" t="s">
+      <c r="L13" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="M13" s="27"/>
+      <c r="M13" s="54"/>
       <c r="N13" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="O13" s="59" t="s">
-        <v>12</v>
-      </c>
+      <c r="O13" s="36" t="s">
+        <v>311</v>
+      </c>
+      <c r="P13" s="72"/>
     </row>
-    <row r="14" spans="1:15" ht="86" customHeight="1">
-      <c r="A14" s="46" t="s">
-        <v>298</v>
-      </c>
-      <c r="B14" s="29"/>
+    <row r="14" spans="1:16" ht="95" customHeight="1">
+      <c r="A14" s="43" t="s">
+        <v>289</v>
+      </c>
+      <c r="B14" s="42"/>
       <c r="C14" s="24" t="s">
         <v>31</v>
       </c>
@@ -2915,13 +3078,13 @@
         <v>32</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F14" s="24" t="s">
         <v>34</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H14" s="24" t="s">
         <v>36</v>
@@ -2944,19 +3107,20 @@
       <c r="N14" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="O14" s="59" t="s">
-        <v>41</v>
-      </c>
+      <c r="O14" s="36" t="s">
+        <v>309</v>
+      </c>
+      <c r="P14" s="72"/>
     </row>
-    <row r="15" spans="1:15" ht="60" customHeight="1">
-      <c r="A15" s="47" t="s">
-        <v>299</v>
+    <row r="15" spans="1:16" ht="48" customHeight="1">
+      <c r="A15" s="46" t="s">
+        <v>290</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D15" s="25" t="s">
         <v>43</v>
@@ -2965,43 +3129,44 @@
         <v>43</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G15" s="25" t="s">
         <v>43</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I15" s="25" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="J15" s="25" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="K15" s="25" t="s">
         <v>49</v>
       </c>
       <c r="L15" s="25" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="M15" s="25" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="N15" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="O15" s="62" t="s">
-        <v>105</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="O15" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="P15" s="72"/>
     </row>
-    <row r="16" spans="1:15" ht="48" customHeight="1">
-      <c r="A16" s="48"/>
+    <row r="16" spans="1:16" ht="48" customHeight="1">
+      <c r="A16" s="47"/>
       <c r="B16" s="26" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D16" s="25" t="s">
         <v>43</v>
@@ -3010,16 +3175,16 @@
         <v>43</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G16" s="25" t="s">
         <v>43</v>
       </c>
       <c r="H16" s="25" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="I16" s="25" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="J16" s="25" t="s">
         <v>55</v>
@@ -3028,22 +3193,23 @@
         <v>44</v>
       </c>
       <c r="L16" s="25" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="M16" s="25" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="N16" s="25" t="s">
-        <v>110</v>
-      </c>
-      <c r="O16" s="60" t="s">
-        <v>111</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="O16" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="P16" s="72"/>
     </row>
-    <row r="17" spans="1:15" ht="75" customHeight="1">
-      <c r="A17" s="48"/>
+    <row r="17" spans="1:16" ht="48" customHeight="1">
+      <c r="A17" s="47"/>
       <c r="B17" s="26" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C17" s="25" t="s">
         <v>50</v>
@@ -3073,22 +3239,23 @@
         <v>62</v>
       </c>
       <c r="L17" s="25" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="M17" s="25" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="N17" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="O17" s="62" t="s">
-        <v>114</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="O17" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="P17" s="72"/>
     </row>
-    <row r="18" spans="1:15" ht="48" customHeight="1">
-      <c r="A18" s="48"/>
+    <row r="18" spans="1:16" ht="48" customHeight="1">
+      <c r="A18" s="47"/>
       <c r="B18" s="26" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C18" s="25" t="s">
         <v>50</v>
@@ -3118,22 +3285,23 @@
         <v>62</v>
       </c>
       <c r="L18" s="25" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="M18" s="25" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="N18" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="O18" s="62" t="s">
-        <v>115</v>
-      </c>
+      <c r="O18" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="P18" s="72"/>
     </row>
-    <row r="19" spans="1:15" ht="75" customHeight="1">
-      <c r="A19" s="48"/>
+    <row r="19" spans="1:16" ht="48" customHeight="1">
+      <c r="A19" s="47"/>
       <c r="B19" s="26" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="C19" s="25" t="s">
         <v>45</v>
@@ -3171,29 +3339,30 @@
       <c r="N19" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="O19" s="62" t="s">
-        <v>116</v>
-      </c>
+      <c r="O19" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="P19" s="72"/>
     </row>
-    <row r="20" spans="1:15" ht="75" customHeight="1">
-      <c r="A20" s="49"/>
+    <row r="20" spans="1:16" ht="48" customHeight="1">
+      <c r="A20" s="48"/>
       <c r="B20" s="26" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="C20" s="25" t="s">
         <v>45</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="F20" s="25" t="s">
         <v>67</v>
       </c>
       <c r="G20" s="25" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="H20" s="25" t="s">
         <v>67</v>
@@ -3202,65 +3371,74 @@
         <v>77</v>
       </c>
       <c r="J20" s="25" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="K20" s="25" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L20" s="25"/>
       <c r="M20" s="25"/>
       <c r="N20" s="25"/>
-      <c r="O20" s="62" t="s">
-        <v>120</v>
-      </c>
+      <c r="O20" s="37" t="s">
+        <v>310</v>
+      </c>
+      <c r="P20" s="72"/>
     </row>
-    <row r="21" spans="1:15" ht="147" customHeight="1" thickBot="1">
-      <c r="A21" s="55" t="s">
-        <v>121</v>
-      </c>
-      <c r="B21" s="56"/>
-      <c r="C21" s="57" t="s">
-        <v>309</v>
-      </c>
-      <c r="D21" s="57" t="s">
-        <v>308</v>
-      </c>
-      <c r="E21" s="57" t="s">
-        <v>307</v>
-      </c>
-      <c r="F21" s="57" t="s">
-        <v>306</v>
-      </c>
-      <c r="G21" s="57" t="s">
-        <v>305</v>
-      </c>
-      <c r="H21" s="57" t="s">
-        <v>304</v>
-      </c>
-      <c r="I21" s="57" t="s">
-        <v>304</v>
-      </c>
-      <c r="J21" s="57" t="s">
-        <v>122</v>
-      </c>
-      <c r="K21" s="57" t="s">
-        <v>123</v>
-      </c>
-      <c r="L21" s="57" t="s">
-        <v>311</v>
-      </c>
-      <c r="M21" s="57" t="s">
-        <v>311</v>
-      </c>
-      <c r="N21" s="57" t="s">
+    <row r="21" spans="1:16" ht="147" customHeight="1" thickBot="1">
+      <c r="A21" s="39" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" s="40"/>
+      <c r="C21" s="27" t="s">
+        <v>300</v>
+      </c>
+      <c r="D21" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>298</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>297</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="H21" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="I21" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="J21" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="K21" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="L21" s="27" t="s">
+        <v>301</v>
+      </c>
+      <c r="M21" s="27" t="s">
+        <v>301</v>
+      </c>
+      <c r="N21" s="27" t="s">
+        <v>302</v>
+      </c>
+      <c r="O21" s="31" t="s">
         <v>312</v>
       </c>
-      <c r="O21" s="63" t="s">
-        <v>310</v>
-      </c>
+      <c r="P21" s="72"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="17">
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="C1:K1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="P2:P11"/>
+    <mergeCell ref="P12:P21"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
@@ -3271,16 +3449,11 @@
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A5:A10"/>
     <mergeCell ref="A15:A20"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="C1:K1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.43307086614173229" right="0.43307086614173229" top="0.55118110236220474" bottom="0.55118110236220474" header="7.874015748031496E-2" footer="7.874015748031496E-2"/>
-  <pageSetup paperSize="9" scale="49" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="52" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3311,796 +3484,796 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="67" customHeight="1" thickBot="1">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="57" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="58"/>
+      <c r="C1" s="69" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" s="70"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="69" t="s">
+        <v>117</v>
+      </c>
+      <c r="G1" s="71"/>
+      <c r="H1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I1" s="69" t="s">
+        <v>119</v>
+      </c>
+      <c r="J1" s="71"/>
+      <c r="K1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="M1" s="69" t="s">
+        <v>122</v>
+      </c>
+      <c r="N1" s="71"/>
+      <c r="O1" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="30" t="s">
+      <c r="Q1" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D1" s="31"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="30" t="s">
+      <c r="R1" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="2" t="s">
+      <c r="S1" s="69" t="s">
         <v>127</v>
       </c>
-      <c r="I1" s="30" t="s">
+      <c r="T1" s="71"/>
+      <c r="U1" s="69" t="s">
         <v>128</v>
       </c>
-      <c r="J1" s="32"/>
-      <c r="K1" s="2" t="s">
+      <c r="V1" s="71"/>
+      <c r="W1" s="69" t="s">
         <v>129</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="X1" s="71"/>
+      <c r="Y1" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="M1" s="30" t="s">
+      <c r="Z1" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="AC1" s="3" t="s">
         <v>134</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="S1" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="T1" s="32"/>
-      <c r="U1" s="30" t="s">
-        <v>137</v>
-      </c>
-      <c r="V1" s="32"/>
-      <c r="W1" s="30" t="s">
-        <v>138</v>
-      </c>
-      <c r="X1" s="32"/>
-      <c r="Y1" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="76" customHeight="1">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="37"/>
+      <c r="B2" s="61"/>
       <c r="C2" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="Q2" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="R2" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="J2" s="5" t="s">
+      <c r="T2" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="U2" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="V2" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="M2" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="N2" s="5" t="s">
+      <c r="W2" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="X2" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="Y2" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="Z2" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="AA2" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="AB2" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="AC2" s="7" t="s">
         <v>157</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="T2" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="U2" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="W2" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="X2" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="Y2" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="Z2" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="AA2" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="AB2" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="AC2" s="7" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="51" customHeight="1">
-      <c r="A3" s="38" t="s">
-        <v>294</v>
-      </c>
-      <c r="B3" s="39"/>
+      <c r="A3" s="62" t="s">
+        <v>285</v>
+      </c>
+      <c r="B3" s="63"/>
       <c r="C3" s="8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="T3" s="8" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="U3" s="8" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="V3" s="8" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="W3" s="8" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="X3" s="8" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="Y3" s="8" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="Z3" s="8" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="AA3" s="8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="AB3" s="8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="AC3" s="9" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="61" customHeight="1">
-      <c r="A4" s="38" t="s">
-        <v>293</v>
-      </c>
-      <c r="B4" s="39"/>
+      <c r="A4" s="62" t="s">
+        <v>284</v>
+      </c>
+      <c r="B4" s="63"/>
       <c r="C4" s="8" t="s">
         <v>48</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>67</v>
       </c>
       <c r="G4" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="P4" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="S4" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="T4" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="U4" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="V4" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="W4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="X4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="Y4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="Z4" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="AA4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="AB4" s="8" t="s">
         <v>176</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="M4" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="N4" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="O4" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="P4" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="Q4" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="R4" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="S4" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="T4" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="U4" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="V4" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="W4" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="X4" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="Y4" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="Z4" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="AA4" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="AB4" s="8" t="s">
-        <v>185</v>
       </c>
       <c r="AC4" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="81" customHeight="1">
-      <c r="A5" s="40" t="s">
-        <v>299</v>
+      <c r="A5" s="64" t="s">
+        <v>290</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>48</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>67</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Q5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="R5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="S5" s="8" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="T5" s="8" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="U5" s="8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="V5" s="8" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="W5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="X5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Y5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Z5" s="8" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="AA5" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AB5" s="8" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="AC5" s="9" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="83" customHeight="1">
-      <c r="A6" s="41"/>
+      <c r="A6" s="65"/>
       <c r="B6" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="N6" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="E6" s="8" t="s">
+      <c r="O6" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="P6" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q6" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="R6" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="S6" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="I6" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="J6" s="8" t="s">
+      <c r="T6" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="K6" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="M6" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="N6" s="8" t="s">
+      <c r="U6" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="V6" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="W6" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="O6" s="8" t="s">
+      <c r="X6" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="Y6" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="Z6" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="AA6" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="P6" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q6" s="10" t="s">
+      <c r="AB6" s="8" t="s">
         <v>156</v>
-      </c>
-      <c r="R6" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="S6" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="T6" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="U6" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="V6" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="W6" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="X6" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="Y6" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="Z6" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="AA6" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="AB6" s="8" t="s">
-        <v>165</v>
       </c>
       <c r="AC6" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:29" ht="83" customHeight="1">
-      <c r="A7" s="41"/>
+      <c r="A7" s="65"/>
       <c r="B7" s="4" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>47</v>
       </c>
       <c r="J7" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="N7" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="P7" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q7" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="R7" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="S7" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="T7" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="K7" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="M7" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="N7" s="8" t="s">
+      <c r="U7" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="V7" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="W7" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="O7" s="8" t="s">
+      <c r="X7" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="Y7" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="Z7" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="AA7" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="P7" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q7" s="10" t="s">
+      <c r="AB7" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="R7" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="S7" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="T7" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="U7" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="V7" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="W7" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="X7" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="Y7" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="Z7" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="AA7" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="AB7" s="8" t="s">
-        <v>165</v>
-      </c>
       <c r="AC7" s="9" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="65" customHeight="1">
-      <c r="A8" s="41"/>
+      <c r="A8" s="65"/>
       <c r="B8" s="4" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>51</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="O8" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="P8" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Q8" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="R8" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="T8" s="8" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="U8" s="8" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="V8" s="8" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="W8" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="X8" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Y8" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Z8" s="8" t="s">
         <v>52</v>
       </c>
       <c r="AA8" s="8" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="AC8" s="9" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="59" customHeight="1" thickBot="1">
-      <c r="A9" s="41"/>
+      <c r="A9" s="65"/>
       <c r="B9" s="11" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="O9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="P9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Q9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="R9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="S9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="T9" s="12" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="U9" s="12" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="V9" s="12" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="W9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="X9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Y9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Z9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AA9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AB9" s="12" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AC9" s="13" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="55" customHeight="1" thickBot="1">
-      <c r="A10" s="42"/>
+      <c r="A10" s="66"/>
       <c r="B10" s="1" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>25</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="F10" s="14" t="s">
         <v>58</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="I10" s="14" t="s">
         <v>60</v>
@@ -4109,34 +4282,34 @@
         <v>61</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="L10" s="14" t="s">
         <v>60</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="N10" s="14" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="O10" s="14" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="P10" s="14" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="Q10" s="14" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="R10" s="14" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="S10" s="14" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="T10" s="14" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="U10" s="14" t="s">
         <v>61</v>
@@ -4145,136 +4318,136 @@
         <v>53</v>
       </c>
       <c r="W10" s="14" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="X10" s="14" t="s">
         <v>59</v>
       </c>
       <c r="Y10" s="14" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="Z10" s="14" t="s">
         <v>44</v>
       </c>
       <c r="AA10" s="14" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="AB10" s="14" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="AC10" s="15" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="53" customHeight="1">
-      <c r="A11" s="36" t="s">
-        <v>295</v>
-      </c>
-      <c r="B11" s="37"/>
+      <c r="A11" s="60" t="s">
+        <v>286</v>
+      </c>
+      <c r="B11" s="61"/>
       <c r="C11" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="I11" s="16" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="J11" s="16" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="K11" s="16" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="O11" s="16" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="Q11" s="16" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="R11" s="16" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="S11" s="16" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="T11" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="U11" s="16" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="V11" s="16" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="W11" s="16" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="X11" s="16" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="Y11" s="16" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="Z11" s="16" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="AA11" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="AB11" s="16" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="AC11" s="17" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="71" customHeight="1">
-      <c r="A12" s="38" t="s">
-        <v>296</v>
-      </c>
-      <c r="B12" s="39"/>
+      <c r="A12" s="62" t="s">
+        <v>287</v>
+      </c>
+      <c r="B12" s="63"/>
       <c r="C12" s="18" t="s">
         <v>48</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="F12" s="18" t="s">
         <v>67</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="I12" s="18" t="s">
         <v>51</v>
@@ -4283,34 +4456,34 @@
         <v>52</v>
       </c>
       <c r="K12" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="L12" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="M12" s="18" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="N12" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="O12" s="18" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="P12" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Q12" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="R12" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="S12" s="18" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="T12" s="19" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="U12" s="18" t="s">
         <v>52</v>
@@ -4319,49 +4492,49 @@
         <v>46</v>
       </c>
       <c r="W12" s="18" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="X12" s="18" t="s">
         <v>47</v>
       </c>
       <c r="Y12" s="18" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="Z12" s="18" t="s">
         <v>48</v>
       </c>
       <c r="AA12" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AB12" s="18" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="AC12" s="20" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:29" ht="81" customHeight="1">
-      <c r="A13" s="38" t="s">
-        <v>297</v>
-      </c>
-      <c r="B13" s="39"/>
+      <c r="A13" s="62" t="s">
+        <v>288</v>
+      </c>
+      <c r="B13" s="63"/>
       <c r="C13" s="18" t="s">
         <v>48</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>67</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="I13" s="18" t="s">
         <v>60</v>
@@ -4370,34 +4543,34 @@
         <v>61</v>
       </c>
       <c r="K13" s="18" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="L13" s="18" t="s">
         <v>60</v>
       </c>
       <c r="M13" s="18" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="O13" s="18" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="P13" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Q13" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="R13" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="S13" s="18" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="T13" s="23" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="U13" s="18" t="s">
         <v>61</v>
@@ -4406,49 +4579,49 @@
         <v>53</v>
       </c>
       <c r="W13" s="18" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="X13" s="18" t="s">
         <v>54</v>
       </c>
       <c r="Y13" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Z13" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AA13" s="18" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AB13" s="18" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="AC13" s="20" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:29" ht="53" customHeight="1">
-      <c r="A14" s="38" t="s">
-        <v>298</v>
-      </c>
-      <c r="B14" s="39"/>
+      <c r="A14" s="62" t="s">
+        <v>289</v>
+      </c>
+      <c r="B14" s="63"/>
       <c r="C14" s="18" t="s">
         <v>25</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="F14" s="18" t="s">
         <v>58</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="I14" s="18" t="s">
         <v>60</v>
@@ -4457,34 +4630,34 @@
         <v>61</v>
       </c>
       <c r="K14" s="18" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="L14" s="18" t="s">
         <v>60</v>
       </c>
       <c r="M14" s="18" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="O14" s="18" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="P14" s="18" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="Q14" s="18" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="R14" s="18" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="S14" s="18" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="T14" s="18" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="U14" s="18" t="s">
         <v>61</v>
@@ -4493,51 +4666,51 @@
         <v>53</v>
       </c>
       <c r="W14" s="18" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="X14" s="18" t="s">
         <v>59</v>
       </c>
       <c r="Y14" s="18" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="Z14" s="18" t="s">
         <v>44</v>
       </c>
       <c r="AA14" s="18" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="AB14" s="18" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="AC14" s="20" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="57.5" customHeight="1">
-      <c r="A15" s="43" t="s">
-        <v>299</v>
+      <c r="A15" s="67" t="s">
+        <v>290</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>64</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="I15" s="18" t="s">
         <v>65</v>
@@ -4546,34 +4719,34 @@
         <v>66</v>
       </c>
       <c r="K15" s="18" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="L15" s="18" t="s">
         <v>65</v>
       </c>
       <c r="M15" s="18" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="O15" s="19" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="P15" s="18" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="Q15" s="18" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="R15" s="18" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="S15" s="18" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="T15" s="23" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="U15" s="18" t="s">
         <v>66</v>
@@ -4582,49 +4755,49 @@
         <v>58</v>
       </c>
       <c r="W15" s="18" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="X15" s="18" t="s">
         <v>63</v>
       </c>
       <c r="Y15" s="18" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="Z15" s="18" t="s">
         <v>55</v>
       </c>
       <c r="AA15" s="18" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="AB15" s="18" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="AC15" s="20" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="71" customHeight="1">
-      <c r="A16" s="44"/>
+      <c r="A16" s="68"/>
       <c r="B16" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>70</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="I16" s="18" t="s">
         <v>72</v>
@@ -4633,34 +4806,34 @@
         <v>73</v>
       </c>
       <c r="K16" s="18" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="L16" s="18" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="M16" s="18" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="N16" s="18" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="O16" s="18" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="P16" s="18" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="Q16" s="18" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="R16" s="18" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="S16" s="18" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="T16" s="19" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="U16" s="18" t="s">
         <v>73</v>
@@ -4669,7 +4842,7 @@
         <v>67</v>
       </c>
       <c r="W16" s="18" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="X16" s="18" t="s">
         <v>69</v>
@@ -4678,40 +4851,40 @@
         <v>71</v>
       </c>
       <c r="Z16" s="18" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="AA16" s="18" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="AB16" s="18" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="AC16" s="20" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" spans="1:29" ht="51" customHeight="1" thickBot="1">
-      <c r="A17" s="44"/>
+      <c r="A17" s="68"/>
       <c r="B17" s="4" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C17" s="21" t="s">
         <v>78</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="H17" s="21" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="I17" s="21" t="s">
         <v>72</v>
@@ -4720,34 +4893,34 @@
         <v>73</v>
       </c>
       <c r="K17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="L17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="M17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="N17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="O17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="P17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Q17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="R17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="S17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="T17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="U17" s="21" t="s">
         <v>73</v>
@@ -4756,51 +4929,58 @@
         <v>67</v>
       </c>
       <c r="W17" s="21" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="X17" s="21" t="s">
         <v>77</v>
       </c>
       <c r="Y17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="Z17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AA17" s="21" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="AB17" s="21" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="AC17" s="22" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="1:29" ht="40">
-      <c r="A18" s="44"/>
+      <c r="A18" s="68"/>
       <c r="B18" s="4" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="20.5" customHeight="1" thickBot="1">
-      <c r="A19" s="44"/>
+      <c r="A19" s="68"/>
       <c r="B19" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20" spans="1:29" ht="40.5" thickBot="1">
-      <c r="A20" s="44"/>
+      <c r="A20" s="68"/>
       <c r="B20" s="1" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
     </row>
     <row r="21" spans="1:29">
-      <c r="A21" s="35"/>
-      <c r="B21" s="35"/>
+      <c r="A21" s="59"/>
+      <c r="B21" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="W1:X1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="S1:T1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A2:B2"/>
@@ -4812,13 +4992,6 @@
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A5:A10"/>
     <mergeCell ref="A15:A20"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="W1:X1"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="S1:T1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
Revise Japanese auxiliary verbs workbook
</commit_message>
<xml_diff>
--- a/Studymaterials/日本語助動詞一覧.xlsx
+++ b/Studymaterials/日本語助動詞一覧.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakag\Desktop\GitHub\Myownproject\Studymaterials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{906E9BDB-44AB-404A-834F-A574DCCA0E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAFB0574-8C6D-48C7-B44C-9B52C83F2189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="316">
   <si>
     <t>品詞</t>
   </si>
@@ -271,9 +271,6 @@
   <si>
     <t>こ
 こよ</t>
-  </si>
-  <si>
-    <t>文語の基本的な動詞活用</t>
   </si>
   <si>
     <t>形容詞ク活用</t>
@@ -1193,6 +1190,16 @@
     <rPh sb="105" eb="107">
       <t>コウセイ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>堂々と　
+　している</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>文語の基本的な
+動詞活用</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1351,7 +1358,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="47">
+  <borders count="49">
     <border>
       <left/>
       <right/>
@@ -1958,16 +1965,44 @@
       <left style="medium">
         <color indexed="8"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
@@ -2081,36 +2116,6 @@
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2129,6 +2134,41 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -2165,13 +2205,14 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2475,50 +2516,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
   <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="9" width="6" customWidth="1"/>
+    <col min="1" max="1" width="4.453125" customWidth="1"/>
+    <col min="2" max="2" width="4.90625" customWidth="1"/>
+    <col min="3" max="9" width="6" customWidth="1"/>
     <col min="10" max="10" width="8" customWidth="1"/>
     <col min="11" max="13" width="6" customWidth="1"/>
     <col min="14" max="14" width="8" customWidth="1"/>
     <col min="15" max="15" width="7.1796875" customWidth="1"/>
-    <col min="16" max="16" width="7.81640625" customWidth="1"/>
+    <col min="16" max="16" width="8.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="24" customHeight="1">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="49" t="s">
+      <c r="B1" s="46"/>
+      <c r="C1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="49" t="s">
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="50"/>
-      <c r="N1" s="49" t="s">
+      <c r="M1" s="40"/>
+      <c r="N1" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="52"/>
+      <c r="O1" s="42"/>
     </row>
     <row r="2" spans="1:16" ht="64" customHeight="1">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="42"/>
+      <c r="B2" s="50"/>
       <c r="C2" s="24" t="s">
         <v>5</v>
       </c>
@@ -2559,14 +2599,14 @@
         <v>17</v>
       </c>
       <c r="P2" s="72" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="82" customHeight="1">
-      <c r="A3" s="43" t="s">
-        <v>285</v>
-      </c>
-      <c r="B3" s="42"/>
+      <c r="A3" s="51" t="s">
+        <v>284</v>
+      </c>
+      <c r="B3" s="50"/>
       <c r="C3" s="24" t="s">
         <v>18</v>
       </c>
@@ -2606,13 +2646,13 @@
       <c r="O3" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="P3" s="72"/>
+      <c r="P3" s="73"/>
     </row>
-    <row r="4" spans="1:16" ht="78" customHeight="1">
-      <c r="A4" s="43" t="s">
-        <v>284</v>
-      </c>
-      <c r="B4" s="42"/>
+    <row r="4" spans="1:16" ht="64" customHeight="1">
+      <c r="A4" s="51" t="s">
+        <v>283</v>
+      </c>
+      <c r="B4" s="50"/>
       <c r="C4" s="24" t="s">
         <v>31</v>
       </c>
@@ -2652,14 +2692,14 @@
       <c r="O4" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="P4" s="72"/>
+      <c r="P4" s="73"/>
     </row>
     <row r="5" spans="1:16" ht="48" customHeight="1">
-      <c r="A5" s="46" t="s">
-        <v>290</v>
+      <c r="A5" s="54" t="s">
+        <v>289</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C5" s="25" t="s">
         <v>42</v>
@@ -2700,12 +2740,12 @@
       <c r="O5" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="P5" s="72"/>
+      <c r="P5" s="73"/>
     </row>
     <row r="6" spans="1:16" ht="48" customHeight="1">
-      <c r="A6" s="47"/>
+      <c r="A6" s="55"/>
       <c r="B6" s="26" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C6" s="25" t="s">
         <v>44</v>
@@ -2746,12 +2786,12 @@
       <c r="O6" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="P6" s="72"/>
+      <c r="P6" s="73"/>
     </row>
     <row r="7" spans="1:16" ht="48" customHeight="1">
-      <c r="A7" s="47"/>
+      <c r="A7" s="55"/>
       <c r="B7" s="26" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>50</v>
@@ -2792,12 +2832,12 @@
       <c r="O7" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="P7" s="72"/>
+      <c r="P7" s="73"/>
     </row>
     <row r="8" spans="1:16" ht="48" customHeight="1">
-      <c r="A8" s="47"/>
+      <c r="A8" s="55"/>
       <c r="B8" s="26" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>50</v>
@@ -2838,12 +2878,12 @@
       <c r="O8" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="P8" s="72"/>
+      <c r="P8" s="73"/>
     </row>
     <row r="9" spans="1:16" ht="48" customHeight="1">
-      <c r="A9" s="47"/>
+      <c r="A9" s="55"/>
       <c r="B9" s="26" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>45</v>
@@ -2884,12 +2924,12 @@
       <c r="O9" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="P9" s="72"/>
+      <c r="P9" s="73"/>
     </row>
     <row r="10" spans="1:16" ht="48" customHeight="1">
-      <c r="A10" s="47"/>
+      <c r="A10" s="55"/>
       <c r="B10" s="33" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C10" s="34" t="s">
         <v>45</v>
@@ -2926,59 +2966,59 @@
       <c r="O10" s="35" t="s">
         <v>73</v>
       </c>
-      <c r="P10" s="72"/>
+      <c r="P10" s="73"/>
     </row>
     <row r="11" spans="1:16" ht="147" customHeight="1" thickBot="1">
-      <c r="A11" s="39" t="s">
-        <v>286</v>
-      </c>
-      <c r="B11" s="40"/>
+      <c r="A11" s="47" t="s">
+        <v>285</v>
+      </c>
+      <c r="B11" s="48"/>
       <c r="C11" s="27" t="s">
+        <v>315</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>303</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="F11" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="G11" s="27" t="s">
+        <v>306</v>
+      </c>
+      <c r="H11" s="27" t="s">
+        <v>302</v>
+      </c>
+      <c r="I11" s="27" t="s">
+        <v>290</v>
+      </c>
+      <c r="J11" s="27" t="s">
+        <v>291</v>
+      </c>
+      <c r="K11" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="L11" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="27" t="s">
-        <v>304</v>
-      </c>
-      <c r="E11" s="27" t="s">
-        <v>306</v>
-      </c>
-      <c r="F11" s="27" t="s">
-        <v>305</v>
-      </c>
-      <c r="G11" s="27" t="s">
-        <v>307</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>303</v>
-      </c>
-      <c r="I11" s="27" t="s">
-        <v>291</v>
-      </c>
-      <c r="J11" s="27" t="s">
-        <v>292</v>
-      </c>
-      <c r="K11" s="27" t="s">
-        <v>308</v>
-      </c>
-      <c r="L11" s="27" t="s">
+      <c r="M11" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="M11" s="27" t="s">
+      <c r="N11" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="N11" s="27" t="s">
+      <c r="O11" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="O11" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="P11" s="72"/>
+      <c r="P11" s="74"/>
     </row>
     <row r="12" spans="1:16" ht="82" customHeight="1">
-      <c r="A12" s="44" t="s">
-        <v>287</v>
-      </c>
-      <c r="B12" s="45"/>
+      <c r="A12" s="52" t="s">
+        <v>286</v>
+      </c>
+      <c r="B12" s="53"/>
       <c r="C12" s="32" t="s">
         <v>18</v>
       </c>
@@ -2986,16 +3026,16 @@
         <v>19</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F12" s="32" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="32" t="s">
         <v>86</v>
-      </c>
-      <c r="H12" s="32" t="s">
-        <v>87</v>
       </c>
       <c r="I12" s="32" t="s">
         <v>24</v>
@@ -3004,31 +3044,31 @@
         <v>64</v>
       </c>
       <c r="K12" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="L12" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="L12" s="32" t="s">
+      <c r="M12" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="M12" s="32" t="s">
+      <c r="N12" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="N12" s="32" t="s">
-        <v>91</v>
-      </c>
       <c r="O12" s="30" t="s">
-        <v>92</v>
+        <v>314</v>
       </c>
       <c r="P12" s="72" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="70" customHeight="1">
-      <c r="A13" s="43" t="s">
-        <v>288</v>
-      </c>
-      <c r="B13" s="42"/>
+      <c r="A13" s="51" t="s">
+        <v>287</v>
+      </c>
+      <c r="B13" s="50"/>
       <c r="C13" s="24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D13" s="24" t="s">
         <v>6</v>
@@ -3037,16 +3077,16 @@
         <v>6</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G13" s="24" t="s">
         <v>8</v>
       </c>
       <c r="H13" s="24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I13" s="24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J13" s="24" t="s">
         <v>12</v>
@@ -3054,23 +3094,23 @@
       <c r="K13" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="L13" s="53" t="s">
+      <c r="L13" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="M13" s="54"/>
+      <c r="M13" s="44"/>
       <c r="N13" s="24" t="s">
         <v>3</v>
       </c>
       <c r="O13" s="36" t="s">
-        <v>311</v>
-      </c>
-      <c r="P13" s="72"/>
+        <v>310</v>
+      </c>
+      <c r="P13" s="73"/>
     </row>
     <row r="14" spans="1:16" ht="95" customHeight="1">
-      <c r="A14" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="B14" s="42"/>
+      <c r="A14" s="51" t="s">
+        <v>288</v>
+      </c>
+      <c r="B14" s="50"/>
       <c r="C14" s="24" t="s">
         <v>31</v>
       </c>
@@ -3078,13 +3118,13 @@
         <v>32</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F14" s="24" t="s">
         <v>34</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H14" s="24" t="s">
         <v>36</v>
@@ -3108,19 +3148,19 @@
         <v>40</v>
       </c>
       <c r="O14" s="36" t="s">
-        <v>309</v>
-      </c>
-      <c r="P14" s="72"/>
+        <v>308</v>
+      </c>
+      <c r="P14" s="73"/>
     </row>
     <row r="15" spans="1:16" ht="48" customHeight="1">
-      <c r="A15" s="46" t="s">
-        <v>290</v>
+      <c r="A15" s="54" t="s">
+        <v>289</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D15" s="25" t="s">
         <v>43</v>
@@ -3129,44 +3169,44 @@
         <v>43</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G15" s="25" t="s">
         <v>43</v>
       </c>
       <c r="H15" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="I15" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="I15" s="25" t="s">
+      <c r="J15" s="25" t="s">
         <v>98</v>
-      </c>
-      <c r="J15" s="25" t="s">
-        <v>99</v>
       </c>
       <c r="K15" s="25" t="s">
         <v>49</v>
       </c>
       <c r="L15" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="M15" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="N15" s="25" t="s">
         <v>100</v>
-      </c>
-      <c r="M15" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="N15" s="25" t="s">
-        <v>101</v>
       </c>
       <c r="O15" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="P15" s="72"/>
+      <c r="P15" s="73"/>
     </row>
     <row r="16" spans="1:16" ht="48" customHeight="1">
-      <c r="A16" s="47"/>
+      <c r="A16" s="55"/>
       <c r="B16" s="26" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D16" s="25" t="s">
         <v>43</v>
@@ -3175,16 +3215,16 @@
         <v>43</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G16" s="25" t="s">
         <v>43</v>
       </c>
       <c r="H16" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="I16" s="25" t="s">
         <v>103</v>
-      </c>
-      <c r="I16" s="25" t="s">
-        <v>104</v>
       </c>
       <c r="J16" s="25" t="s">
         <v>55</v>
@@ -3193,23 +3233,23 @@
         <v>44</v>
       </c>
       <c r="L16" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="M16" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="N16" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="N16" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="O16" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="P16" s="72"/>
+      <c r="P16" s="73"/>
     </row>
     <row r="17" spans="1:16" ht="48" customHeight="1">
-      <c r="A17" s="47"/>
+      <c r="A17" s="55"/>
       <c r="B17" s="26" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C17" s="25" t="s">
         <v>50</v>
@@ -3239,23 +3279,23 @@
         <v>62</v>
       </c>
       <c r="L17" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="M17" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="N17" s="25" t="s">
         <v>107</v>
-      </c>
-      <c r="M17" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="N17" s="25" t="s">
-        <v>108</v>
       </c>
       <c r="O17" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="P17" s="72"/>
+      <c r="P17" s="73"/>
     </row>
     <row r="18" spans="1:16" ht="48" customHeight="1">
-      <c r="A18" s="47"/>
+      <c r="A18" s="55"/>
       <c r="B18" s="26" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C18" s="25" t="s">
         <v>50</v>
@@ -3285,10 +3325,10 @@
         <v>62</v>
       </c>
       <c r="L18" s="25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M18" s="25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="N18" s="25" t="s">
         <v>47</v>
@@ -3296,12 +3336,12 @@
       <c r="O18" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="P18" s="72"/>
+      <c r="P18" s="73"/>
     </row>
     <row r="19" spans="1:16" ht="48" customHeight="1">
-      <c r="A19" s="47"/>
+      <c r="A19" s="55"/>
       <c r="B19" s="26" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C19" s="25" t="s">
         <v>45</v>
@@ -3342,27 +3382,27 @@
       <c r="O19" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="P19" s="72"/>
+      <c r="P19" s="73"/>
     </row>
     <row r="20" spans="1:16" ht="48" customHeight="1">
-      <c r="A20" s="48"/>
+      <c r="A20" s="56"/>
       <c r="B20" s="26" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C20" s="25" t="s">
         <v>45</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F20" s="25" t="s">
         <v>67</v>
       </c>
       <c r="G20" s="25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H20" s="25" t="s">
         <v>67</v>
@@ -3371,72 +3411,67 @@
         <v>77</v>
       </c>
       <c r="J20" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="K20" s="25" t="s">
         <v>110</v>
-      </c>
-      <c r="K20" s="25" t="s">
-        <v>111</v>
       </c>
       <c r="L20" s="25"/>
       <c r="M20" s="25"/>
       <c r="N20" s="25"/>
       <c r="O20" s="37" t="s">
-        <v>310</v>
-      </c>
-      <c r="P20" s="72"/>
+        <v>309</v>
+      </c>
+      <c r="P20" s="73"/>
     </row>
     <row r="21" spans="1:16" ht="147" customHeight="1" thickBot="1">
-      <c r="A21" s="39" t="s">
+      <c r="A21" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="B21" s="48"/>
+      <c r="C21" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="D21" s="27" t="s">
+        <v>298</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>297</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="H21" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="I21" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="J21" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="27" t="s">
+      <c r="K21" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="L21" s="27" t="s">
         <v>300</v>
       </c>
-      <c r="D21" s="27" t="s">
-        <v>299</v>
-      </c>
-      <c r="E21" s="27" t="s">
-        <v>298</v>
-      </c>
-      <c r="F21" s="27" t="s">
-        <v>297</v>
-      </c>
-      <c r="G21" s="27" t="s">
-        <v>296</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>295</v>
-      </c>
-      <c r="I21" s="27" t="s">
-        <v>295</v>
-      </c>
-      <c r="J21" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="K21" s="27" t="s">
-        <v>114</v>
-      </c>
-      <c r="L21" s="27" t="s">
+      <c r="M21" s="27" t="s">
+        <v>300</v>
+      </c>
+      <c r="N21" s="27" t="s">
         <v>301</v>
       </c>
-      <c r="M21" s="27" t="s">
-        <v>301</v>
-      </c>
-      <c r="N21" s="27" t="s">
-        <v>302</v>
-      </c>
       <c r="O21" s="31" t="s">
-        <v>312</v>
-      </c>
-      <c r="P21" s="72"/>
+        <v>311</v>
+      </c>
+      <c r="P21" s="74"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="C1:K1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="A1:B1"/>
     <mergeCell ref="P2:P11"/>
     <mergeCell ref="P12:P21"/>
     <mergeCell ref="A21:B21"/>
@@ -3449,11 +3484,16 @@
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A5:A10"/>
     <mergeCell ref="A15:A20"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="C1:K1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.43307086614173229" right="0.43307086614173229" top="0.55118110236220474" bottom="0.55118110236220474" header="7.874015748031496E-2" footer="7.874015748031496E-2"/>
-  <pageSetup paperSize="9" scale="52" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="59" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3484,796 +3524,796 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="67" customHeight="1" thickBot="1">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="61"/>
+      <c r="C1" s="57" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="69" t="s">
+      <c r="D1" s="58"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="57" t="s">
         <v>116</v>
       </c>
-      <c r="D1" s="70"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="69" t="s">
+      <c r="G1" s="59"/>
+      <c r="H1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G1" s="71"/>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="57" t="s">
         <v>118</v>
       </c>
-      <c r="I1" s="69" t="s">
+      <c r="J1" s="59"/>
+      <c r="K1" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="J1" s="71"/>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="57" t="s">
         <v>121</v>
       </c>
-      <c r="M1" s="69" t="s">
+      <c r="N1" s="59"/>
+      <c r="O1" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="N1" s="71"/>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="57" t="s">
         <v>126</v>
       </c>
-      <c r="S1" s="69" t="s">
+      <c r="T1" s="59"/>
+      <c r="U1" s="57" t="s">
         <v>127</v>
       </c>
-      <c r="T1" s="71"/>
-      <c r="U1" s="69" t="s">
+      <c r="V1" s="59"/>
+      <c r="W1" s="57" t="s">
         <v>128</v>
       </c>
-      <c r="V1" s="71"/>
-      <c r="W1" s="69" t="s">
+      <c r="X1" s="59"/>
+      <c r="Y1" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="X1" s="71"/>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="3" t="s">
         <v>133</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="76" customHeight="1">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="61"/>
+      <c r="B2" s="64"/>
       <c r="C2" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="J2" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="M2" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="Q2" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="R2" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="S2" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="T2" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="U2" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="V2" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="V2" s="5" t="s">
+      <c r="W2" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="W2" s="5" t="s">
+      <c r="X2" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="Y2" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="X2" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="Y2" s="5" t="s">
+      <c r="Z2" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA2" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="Z2" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA2" s="6" t="s">
+      <c r="AB2" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="AB2" s="5" t="s">
+      <c r="AC2" s="7" t="s">
         <v>156</v>
-      </c>
-      <c r="AC2" s="7" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="51" customHeight="1">
-      <c r="A3" s="62" t="s">
-        <v>285</v>
-      </c>
-      <c r="B3" s="63"/>
+      <c r="A3" s="65" t="s">
+        <v>284</v>
+      </c>
+      <c r="B3" s="66"/>
       <c r="C3" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="I3" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q3" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="R3" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="S3" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="T3" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="U3" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="V3" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="W3" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="K3" s="8" t="s">
+      <c r="X3" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="Y3" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="Z3" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA3" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB3" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="AC3" s="9" t="s">
         <v>161</v>
-      </c>
-      <c r="L3" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="O3" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="P3" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="Q3" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="R3" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="S3" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="T3" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="U3" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="V3" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="W3" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="X3" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="Y3" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="Z3" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="AA3" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="AB3" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="AC3" s="9" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="61" customHeight="1">
-      <c r="A4" s="62" t="s">
-        <v>284</v>
-      </c>
-      <c r="B4" s="63"/>
+      <c r="A4" s="65" t="s">
+        <v>283</v>
+      </c>
+      <c r="B4" s="66"/>
       <c r="C4" s="8" t="s">
         <v>48</v>
       </c>
       <c r="D4" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>164</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>165</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>67</v>
       </c>
       <c r="G4" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="H4" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="H4" s="8" t="s">
-        <v>167</v>
-      </c>
       <c r="I4" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="K4" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="L4" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="M4" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="N4" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="M4" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="N4" s="8" t="s">
+      <c r="O4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="P4" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="S4" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="O4" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="P4" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="Q4" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="R4" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="S4" s="8" t="s">
+      <c r="T4" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="T4" s="8" t="s">
+      <c r="U4" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="V4" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="U4" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="V4" s="8" t="s">
+      <c r="W4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="X4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="Y4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="Z4" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="W4" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="X4" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="Y4" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="Z4" s="8" t="s">
+      <c r="AA4" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB4" s="8" t="s">
         <v>175</v>
-      </c>
-      <c r="AA4" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="AB4" s="8" t="s">
-        <v>176</v>
       </c>
       <c r="AC4" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="81" customHeight="1">
-      <c r="A5" s="64" t="s">
-        <v>290</v>
+      <c r="A5" s="67" t="s">
+        <v>289</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>48</v>
       </c>
       <c r="D5" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>164</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>165</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>67</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H5" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="K5" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="M5" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="N5" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="M5" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="N5" s="8" t="s">
+      <c r="O5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="R5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="S5" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="O5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="P5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="Q5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="R5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="S5" s="8" t="s">
+      <c r="T5" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="T5" s="8" t="s">
+      <c r="U5" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="V5" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="U5" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="V5" s="8" t="s">
+      <c r="W5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="X5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="Y5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="Z5" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA5" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB5" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="W5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="X5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="Y5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="Z5" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA5" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="AB5" s="8" t="s">
-        <v>185</v>
-      </c>
       <c r="AC5" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="83" customHeight="1">
-      <c r="A6" s="65"/>
+      <c r="A6" s="68"/>
       <c r="B6" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="E6" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="G6" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="H6" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="I6" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="J6" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="I6" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="J6" s="8" t="s">
+      <c r="K6" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="L6" s="8" t="s">
+      <c r="M6" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="N6" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="M6" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="N6" s="8" t="s">
-        <v>144</v>
-      </c>
       <c r="O6" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="P6" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q6" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="P6" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="Q6" s="10" t="s">
+      <c r="R6" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="R6" s="10" t="s">
+      <c r="S6" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="S6" s="8" t="s">
+      <c r="T6" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="T6" s="8" t="s">
-        <v>150</v>
-      </c>
       <c r="U6" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="V6" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="W6" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="X6" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="Y6" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="X6" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="Y6" s="8" t="s">
+      <c r="Z6" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA6" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="Z6" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA6" s="10" t="s">
+      <c r="AB6" s="8" t="s">
         <v>155</v>
-      </c>
-      <c r="AB6" s="8" t="s">
-        <v>156</v>
       </c>
       <c r="AC6" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:29" ht="83" customHeight="1">
-      <c r="A7" s="65"/>
+      <c r="A7" s="68"/>
       <c r="B7" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>140</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>47</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K7" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="L7" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="L7" s="8" t="s">
-        <v>188</v>
-      </c>
       <c r="M7" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O7" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="P7" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q7" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="P7" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="Q7" s="10" t="s">
+      <c r="R7" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="R7" s="10" t="s">
+      <c r="S7" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="S7" s="8" t="s">
+      <c r="T7" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="T7" s="8" t="s">
-        <v>150</v>
-      </c>
       <c r="U7" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="V7" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="W7" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="X7" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="Y7" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="X7" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="Y7" s="8" t="s">
+      <c r="Z7" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA7" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="Z7" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA7" s="10" t="s">
+      <c r="AB7" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="AB7" s="8" t="s">
-        <v>156</v>
-      </c>
       <c r="AC7" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="65" customHeight="1">
-      <c r="A8" s="65"/>
+      <c r="A8" s="68"/>
       <c r="B8" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C8" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="G8" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="H8" s="8" t="s">
         <v>193</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>194</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>51</v>
       </c>
       <c r="J8" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="K8" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="L8" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="M8" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="N8" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="M8" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="N8" s="10" t="s">
+      <c r="O8" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="P8" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q8" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="R8" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="S8" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="O8" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="P8" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="Q8" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="R8" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="S8" s="8" t="s">
+      <c r="T8" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="T8" s="8" t="s">
+      <c r="U8" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="U8" s="8" t="s">
+      <c r="V8" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="V8" s="8" t="s">
-        <v>202</v>
-      </c>
       <c r="W8" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="X8" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Y8" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Z8" s="8" t="s">
         <v>52</v>
       </c>
       <c r="AA8" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AC8" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="59" customHeight="1" thickBot="1">
-      <c r="A9" s="65"/>
+      <c r="A9" s="68"/>
       <c r="B9" s="11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C9" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="E9" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="F9" s="12" t="s">
         <v>206</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="G9" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="H9" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="I9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="K9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="L9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="M9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="N9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="O9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="P9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="R9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="S9" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="T9" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="U9" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="I9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="J9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="K9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="L9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="M9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="N9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="O9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="P9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="Q9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="R9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="S9" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="T9" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="U9" s="12" t="s">
-        <v>210</v>
-      </c>
       <c r="V9" s="12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="W9" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="X9" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Y9" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Z9" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AA9" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AB9" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AC9" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="55" customHeight="1" thickBot="1">
-      <c r="A10" s="66"/>
+      <c r="A10" s="69"/>
       <c r="B10" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>25</v>
       </c>
       <c r="D10" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>211</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>212</v>
       </c>
       <c r="F10" s="14" t="s">
         <v>58</v>
       </c>
       <c r="G10" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="H10" s="14" t="s">
         <v>213</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>214</v>
       </c>
       <c r="I10" s="14" t="s">
         <v>60</v>
@@ -4282,34 +4322,34 @@
         <v>61</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="L10" s="14" t="s">
         <v>60</v>
       </c>
       <c r="M10" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="N10" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="N10" s="14" t="s">
+      <c r="O10" s="14" t="s">
         <v>217</v>
       </c>
-      <c r="O10" s="14" t="s">
+      <c r="P10" s="14" t="s">
         <v>218</v>
       </c>
-      <c r="P10" s="14" t="s">
+      <c r="Q10" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="Q10" s="14" t="s">
+      <c r="R10" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="R10" s="14" t="s">
+      <c r="S10" s="14" t="s">
         <v>221</v>
       </c>
-      <c r="S10" s="14" t="s">
+      <c r="T10" s="14" t="s">
         <v>222</v>
-      </c>
-      <c r="T10" s="14" t="s">
-        <v>223</v>
       </c>
       <c r="U10" s="14" t="s">
         <v>61</v>
@@ -4318,136 +4358,136 @@
         <v>53</v>
       </c>
       <c r="W10" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="X10" s="14" t="s">
         <v>59</v>
       </c>
       <c r="Y10" s="14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="Z10" s="14" t="s">
         <v>44</v>
       </c>
       <c r="AA10" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB10" s="14" t="s">
         <v>226</v>
-      </c>
-      <c r="AB10" s="14" t="s">
-        <v>227</v>
       </c>
       <c r="AC10" s="15" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="53" customHeight="1">
-      <c r="A11" s="60" t="s">
-        <v>286</v>
-      </c>
-      <c r="B11" s="61"/>
+      <c r="A11" s="63" t="s">
+        <v>285</v>
+      </c>
+      <c r="B11" s="64"/>
       <c r="C11" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="I11" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="J11" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="N11" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="O11" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="P11" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q11" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="R11" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="D11" s="16" t="s">
-        <v>276</v>
-      </c>
-      <c r="E11" s="16" t="s">
+      <c r="S11" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="T11" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="U11" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="V11" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="W11" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="H11" s="16" t="s">
-        <v>293</v>
-      </c>
-      <c r="I11" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="J11" s="16" t="s">
-        <v>292</v>
-      </c>
-      <c r="K11" s="16" t="s">
+      <c r="X11" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="Y11" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="Z11" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="AA11" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB11" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="AC11" s="17" t="s">
         <v>161</v>
-      </c>
-      <c r="L11" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="M11" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="N11" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="O11" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="P11" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q11" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="R11" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="S11" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="T11" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="U11" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="V11" s="16" t="s">
-        <v>228</v>
-      </c>
-      <c r="W11" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="X11" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="Y11" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="Z11" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="AA11" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="AB11" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="AC11" s="17" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="71" customHeight="1">
-      <c r="A12" s="62" t="s">
-        <v>287</v>
-      </c>
-      <c r="B12" s="63"/>
+      <c r="A12" s="65" t="s">
+        <v>286</v>
+      </c>
+      <c r="B12" s="66"/>
       <c r="C12" s="18" t="s">
         <v>48</v>
       </c>
       <c r="D12" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="E12" s="18" t="s">
         <v>164</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>165</v>
       </c>
       <c r="F12" s="18" t="s">
         <v>67</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I12" s="18" t="s">
         <v>51</v>
@@ -4456,34 +4496,34 @@
         <v>52</v>
       </c>
       <c r="K12" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="L12" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M12" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="N12" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="O12" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="P12" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q12" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="R12" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="S12" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="N12" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="O12" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="P12" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="Q12" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="R12" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="S12" s="18" t="s">
+      <c r="T12" s="19" t="s">
         <v>231</v>
-      </c>
-      <c r="T12" s="19" t="s">
-        <v>232</v>
       </c>
       <c r="U12" s="18" t="s">
         <v>52</v>
@@ -4492,49 +4532,49 @@
         <v>46</v>
       </c>
       <c r="W12" s="18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="X12" s="18" t="s">
         <v>47</v>
       </c>
       <c r="Y12" s="18" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="Z12" s="18" t="s">
         <v>48</v>
       </c>
       <c r="AA12" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AB12" s="18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AC12" s="20" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:29" ht="81" customHeight="1">
-      <c r="A13" s="62" t="s">
-        <v>288</v>
-      </c>
-      <c r="B13" s="63"/>
+      <c r="A13" s="65" t="s">
+        <v>287</v>
+      </c>
+      <c r="B13" s="66"/>
       <c r="C13" s="18" t="s">
         <v>48</v>
       </c>
       <c r="D13" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="E13" s="18" t="s">
         <v>164</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>165</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>67</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I13" s="18" t="s">
         <v>60</v>
@@ -4543,34 +4583,34 @@
         <v>61</v>
       </c>
       <c r="K13" s="18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="L13" s="18" t="s">
         <v>60</v>
       </c>
       <c r="M13" s="18" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O13" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="P13" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q13" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="R13" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="S13" s="18" t="s">
         <v>238</v>
       </c>
-      <c r="P13" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="Q13" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="R13" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="S13" s="18" t="s">
+      <c r="T13" s="23" t="s">
         <v>239</v>
-      </c>
-      <c r="T13" s="23" t="s">
-        <v>240</v>
       </c>
       <c r="U13" s="18" t="s">
         <v>61</v>
@@ -4579,49 +4619,49 @@
         <v>53</v>
       </c>
       <c r="W13" s="18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="X13" s="18" t="s">
         <v>54</v>
       </c>
       <c r="Y13" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Z13" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AA13" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AB13" s="18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AC13" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:29" ht="53" customHeight="1">
-      <c r="A14" s="62" t="s">
-        <v>289</v>
-      </c>
-      <c r="B14" s="63"/>
+      <c r="A14" s="65" t="s">
+        <v>288</v>
+      </c>
+      <c r="B14" s="66"/>
       <c r="C14" s="18" t="s">
         <v>25</v>
       </c>
       <c r="D14" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="E14" s="18" t="s">
         <v>211</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>212</v>
       </c>
       <c r="F14" s="18" t="s">
         <v>58</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I14" s="18" t="s">
         <v>60</v>
@@ -4630,34 +4670,34 @@
         <v>61</v>
       </c>
       <c r="K14" s="18" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="L14" s="18" t="s">
         <v>60</v>
       </c>
       <c r="M14" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="N14" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="N14" s="18" t="s">
+      <c r="O14" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="O14" s="18" t="s">
+      <c r="P14" s="18" t="s">
         <v>218</v>
       </c>
-      <c r="P14" s="18" t="s">
+      <c r="Q14" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="Q14" s="18" t="s">
+      <c r="R14" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="R14" s="18" t="s">
+      <c r="S14" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="S14" s="18" t="s">
+      <c r="T14" s="18" t="s">
         <v>222</v>
-      </c>
-      <c r="T14" s="18" t="s">
-        <v>223</v>
       </c>
       <c r="U14" s="18" t="s">
         <v>61</v>
@@ -4666,51 +4706,51 @@
         <v>53</v>
       </c>
       <c r="W14" s="18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="X14" s="18" t="s">
         <v>59</v>
       </c>
       <c r="Y14" s="18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="Z14" s="18" t="s">
         <v>44</v>
       </c>
       <c r="AA14" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB14" s="18" t="s">
         <v>226</v>
-      </c>
-      <c r="AB14" s="18" t="s">
-        <v>227</v>
       </c>
       <c r="AC14" s="20" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="57.5" customHeight="1">
-      <c r="A15" s="67" t="s">
-        <v>290</v>
+      <c r="A15" s="70" t="s">
+        <v>289</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>64</v>
       </c>
       <c r="D15" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="E15" s="18" t="s">
         <v>243</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="F15" s="18" t="s">
         <v>244</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="G15" s="18" t="s">
         <v>245</v>
       </c>
-      <c r="G15" s="18" t="s">
-        <v>246</v>
-      </c>
       <c r="H15" s="18" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I15" s="18" t="s">
         <v>65</v>
@@ -4719,34 +4759,34 @@
         <v>66</v>
       </c>
       <c r="K15" s="18" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L15" s="18" t="s">
         <v>65</v>
       </c>
       <c r="M15" s="18" t="s">
+        <v>247</v>
+      </c>
+      <c r="N15" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="O15" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="N15" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="O15" s="19" t="s">
+      <c r="P15" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q15" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="R15" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="S15" s="18" t="s">
         <v>249</v>
       </c>
-      <c r="P15" s="18" t="s">
-        <v>219</v>
-      </c>
-      <c r="Q15" s="18" t="s">
-        <v>220</v>
-      </c>
-      <c r="R15" s="18" t="s">
-        <v>221</v>
-      </c>
-      <c r="S15" s="18" t="s">
+      <c r="T15" s="23" t="s">
         <v>250</v>
-      </c>
-      <c r="T15" s="23" t="s">
-        <v>251</v>
       </c>
       <c r="U15" s="18" t="s">
         <v>66</v>
@@ -4755,49 +4795,49 @@
         <v>58</v>
       </c>
       <c r="W15" s="18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="X15" s="18" t="s">
         <v>63</v>
       </c>
       <c r="Y15" s="18" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="Z15" s="18" t="s">
         <v>55</v>
       </c>
       <c r="AA15" s="18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AB15" s="18" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="AC15" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="71" customHeight="1">
-      <c r="A16" s="68"/>
+      <c r="A16" s="71"/>
       <c r="B16" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>70</v>
       </c>
       <c r="D16" s="18" t="s">
+        <v>254</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>255</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>256</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="G16" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="H16" s="18" t="s">
         <v>258</v>
-      </c>
-      <c r="H16" s="18" t="s">
-        <v>259</v>
       </c>
       <c r="I16" s="18" t="s">
         <v>72</v>
@@ -4806,34 +4846,34 @@
         <v>73</v>
       </c>
       <c r="K16" s="18" t="s">
+        <v>259</v>
+      </c>
+      <c r="L16" s="18" t="s">
+        <v>293</v>
+      </c>
+      <c r="M16" s="18" t="s">
         <v>260</v>
       </c>
-      <c r="L16" s="18" t="s">
-        <v>294</v>
-      </c>
-      <c r="M16" s="18" t="s">
+      <c r="N16" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="O16" s="18" t="s">
         <v>261</v>
       </c>
-      <c r="N16" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="O16" s="18" t="s">
+      <c r="P16" s="18" t="s">
         <v>262</v>
       </c>
-      <c r="P16" s="18" t="s">
+      <c r="Q16" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="Q16" s="18" t="s">
+      <c r="R16" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="R16" s="18" t="s">
+      <c r="S16" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="T16" s="19" t="s">
         <v>265</v>
-      </c>
-      <c r="S16" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="T16" s="19" t="s">
-        <v>266</v>
       </c>
       <c r="U16" s="18" t="s">
         <v>73</v>
@@ -4842,7 +4882,7 @@
         <v>67</v>
       </c>
       <c r="W16" s="18" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="X16" s="18" t="s">
         <v>69</v>
@@ -4851,40 +4891,40 @@
         <v>71</v>
       </c>
       <c r="Z16" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="AA16" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB16" s="18" t="s">
         <v>268</v>
       </c>
-      <c r="AA16" s="18" t="s">
-        <v>226</v>
-      </c>
-      <c r="AB16" s="18" t="s">
-        <v>269</v>
-      </c>
       <c r="AC16" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="1:29" ht="51" customHeight="1" thickBot="1">
-      <c r="A17" s="68"/>
+      <c r="A17" s="71"/>
       <c r="B17" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C17" s="21" t="s">
         <v>78</v>
       </c>
       <c r="D17" s="21" t="s">
+        <v>269</v>
+      </c>
+      <c r="E17" s="21" t="s">
         <v>270</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="F17" s="21" t="s">
         <v>271</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="G17" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="G17" s="21" t="s">
-        <v>273</v>
-      </c>
       <c r="H17" s="21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I17" s="21" t="s">
         <v>72</v>
@@ -4893,34 +4933,34 @@
         <v>73</v>
       </c>
       <c r="K17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="L17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="P17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="R17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="S17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U17" s="21" t="s">
         <v>73</v>
@@ -4929,58 +4969,51 @@
         <v>67</v>
       </c>
       <c r="W17" s="21" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="X17" s="21" t="s">
         <v>77</v>
       </c>
       <c r="Y17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Z17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AA17" s="21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AB17" s="21" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="AC17" s="22" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:29" ht="40">
-      <c r="A18" s="68"/>
+      <c r="A18" s="71"/>
       <c r="B18" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="20.5" customHeight="1" thickBot="1">
-      <c r="A19" s="68"/>
+      <c r="A19" s="71"/>
       <c r="B19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="20" spans="1:29" ht="40.5" thickBot="1">
-      <c r="A20" s="68"/>
+      <c r="A20" s="71"/>
       <c r="B20" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="21" spans="1:29">
-      <c r="A21" s="59"/>
-      <c r="B21" s="59"/>
+      <c r="A21" s="62"/>
+      <c r="B21" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="W1:X1"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="S1:T1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A2:B2"/>
@@ -4992,6 +5025,13 @@
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A5:A10"/>
     <mergeCell ref="A15:A20"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="W1:X1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="S1:T1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>